<commit_message>
data: hourly update 2026-07-13 08:21Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-13.xlsx
+++ b/data/output/workbook/2026-07-13.xlsx
@@ -363,7 +363,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12649200"/>
+    <ext cx="10125075" cy="12877800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 00:34</t>
+          <t>2026-07-13 04:21</t>
         </is>
       </c>
     </row>
@@ -1179,12 +1179,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5547</v>
+        <v>0.5438</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-125</v>
+        <v>-119</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1306,37 +1306,37 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Atlanta Dream</t>
+          <t>Portland Fire @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Connecticut Sun</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5299</v>
+        <v>0.5574</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-113</v>
+        <v>-126</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-104</v>
+        <v>-112</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 55.7% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1396,13 +1396,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5175</v>
+        <v>0.5187</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-107</v>
+        <v>-108</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -2000,17 +2000,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 180.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5299</v>
+        <v>0.5316474443436277</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-113</v>
+        <v>-114</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-104</v>
+        <v>106</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -2066,17 +2066,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 179.5</t>
+          <t>Under 180.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4701</v>
+        <v>0.4683525556563723</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 47.0% (fair +113). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2208,7 +2208,7 @@
         <v>-138</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2400,13 +2400,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5175</v>
+        <v>0.5187</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-107</v>
+        <v>-108</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2466,10 +2466,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4825</v>
+        <v>0.4813</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>104</v>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.3% (fair +107). Your call.</t>
+          <t>Model 48.1% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2604,7 +2604,7 @@
         <v>-115</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -2664,13 +2664,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4453</v>
+        <v>0.4426</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +125). Your call.</t>
+          <t>Model 44.3% (fair +126). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -2730,13 +2730,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5547</v>
+        <v>0.5574</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-125</v>
+        <v>-126</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-105</v>
+        <v>-112</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 55.7% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -2928,13 +2928,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4935</v>
+        <v>0.4965</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +103). Your call.</t>
+          <t>Model 49.6% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -2994,10 +2994,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5065</v>
+        <v>0.5035000000000001</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-103</v>
+        <v>-101</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>100</v>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -103). Your call.</t>
+          <t>Model 50.4% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -3060,13 +3060,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.41237</v>
+        <v>0.4562</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 41.2% (fair +143). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -3126,10 +3126,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.58763</v>
+        <v>0.5438</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-143</v>
+        <v>-119</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>100</v>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 58.8% (fair -143). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -5873,7 +5873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q109"/>
+  <dimension ref="A1:Q111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5890,245 +5890,127 @@
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="29" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
         <is>
           <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="30" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B80" s="30" t="inlineStr">
+      <c r="B82" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C80" s="30" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D80" s="30" t="inlineStr">
+      <c r="D82" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E80" s="30" t="inlineStr">
+      <c r="E82" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F80" s="30" t="inlineStr">
+      <c r="F82" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G80" s="30" t="inlineStr">
+      <c r="G82" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H80" s="30" t="inlineStr">
+      <c r="H82" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I80" s="30" t="inlineStr">
+      <c r="I82" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J80" s="30" t="inlineStr">
+      <c r="J82" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K80" s="30" t="inlineStr">
+      <c r="K82" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L80" s="30" t="inlineStr">
+      <c r="L82" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M80" s="30" t="inlineStr">
+      <c r="M82" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N80" s="30" t="inlineStr">
+      <c r="N82" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O80" s="30" t="inlineStr">
+      <c r="O82" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P80" s="30" t="inlineStr">
+      <c r="P82" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q80" s="30" t="inlineStr">
+      <c r="Q82" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="31" t="inlineStr">
-        <is>
-          <t>PPG</t>
-        </is>
-      </c>
-      <c r="B81" s="32" t="n">
-        <v>83</v>
-      </c>
-      <c r="C81" s="32" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="D81" s="32" t="n">
-        <v>83.05</v>
-      </c>
-      <c r="E81" s="32" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="F81" s="32" t="n">
-        <v>83</v>
-      </c>
-      <c r="G81" s="32" t="n">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="H81" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K81" s="32" t="n">
-        <v>72.75</v>
-      </c>
-      <c r="L81" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="M81" s="32" t="n">
-        <v>80</v>
-      </c>
-      <c r="N81" s="32" t="n">
-        <v>78.72199999999999</v>
-      </c>
-      <c r="O81" s="32" t="n">
-        <v>79</v>
-      </c>
-      <c r="P81" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="Q81" s="34" t="inlineStr">
-        <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B82" s="32" t="n">
-        <v>101.929</v>
-      </c>
-      <c r="C82" s="32" t="n">
-        <v>102.13</v>
-      </c>
-      <c r="D82" s="32" t="n">
-        <v>101.973</v>
-      </c>
-      <c r="E82" s="32" t="n">
-        <v>102.639</v>
-      </c>
-      <c r="F82" s="32" t="n">
-        <v>101.929</v>
-      </c>
-      <c r="G82" s="32" t="n">
-        <v>97.006</v>
-      </c>
-      <c r="H82" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="n">
-        <v>88.01600000000001</v>
-      </c>
-      <c r="L82" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="M82" s="32" t="n">
-        <v>97.129</v>
-      </c>
-      <c r="N82" s="32" t="n">
-        <v>96.706</v>
-      </c>
-      <c r="O82" s="32" t="n">
-        <v>98.628</v>
-      </c>
-      <c r="P82" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="Q82" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>0.476</v>
+        <v>83</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>0.491</v>
+        <v>82.3</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>0.486</v>
+        <v>83.05</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>0.488</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>0.476</v>
+        <v>83</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>0.453</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="H83" s="36" t="inlineStr">
         <is>
-          <t>12th</t>
+          <t>11th</t>
         </is>
       </c>
       <c r="I83" s="32" t="inlineStr"/>
@@ -6138,56 +6020,56 @@
         </is>
       </c>
       <c r="K83" s="32" t="n">
-        <v>0.408</v>
+        <v>72.75</v>
       </c>
       <c r="L83" s="32" t="n">
-        <v>0.441</v>
+        <v>79.75</v>
       </c>
       <c r="M83" s="32" t="n">
-        <v>0.461</v>
+        <v>80</v>
       </c>
       <c r="N83" s="32" t="n">
-        <v>0.464</v>
+        <v>78.72199999999999</v>
       </c>
       <c r="O83" s="32" t="n">
-        <v>0.481</v>
+        <v>79</v>
       </c>
       <c r="P83" s="32" t="n">
-        <v>0.441</v>
+        <v>79.75</v>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>0.467</v>
+        <v>101.929</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>0.48</v>
+        <v>102.13</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>0.486</v>
+        <v>101.973</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>0.488</v>
+        <v>102.639</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>0.467</v>
+        <v>101.929</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>0.454</v>
+        <v>97.006</v>
       </c>
       <c r="H84" s="36" t="inlineStr">
         <is>
-          <t>12th</t>
+          <t>11th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
@@ -6197,52 +6079,52 @@
         </is>
       </c>
       <c r="K84" s="32" t="n">
-        <v>0.404</v>
+        <v>88.01600000000001</v>
       </c>
       <c r="L84" s="32" t="n">
-        <v>0.449</v>
+        <v>95.66500000000001</v>
       </c>
       <c r="M84" s="32" t="n">
-        <v>0.456</v>
+        <v>97.129</v>
       </c>
       <c r="N84" s="32" t="n">
-        <v>0.463</v>
+        <v>96.706</v>
       </c>
       <c r="O84" s="32" t="n">
-        <v>0.461</v>
+        <v>98.628</v>
       </c>
       <c r="P84" s="32" t="n">
-        <v>0.449</v>
+        <v>95.66500000000001</v>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>0.32</v>
+        <v>0.476</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>0.33</v>
+        <v>0.491</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>0.315</v>
+        <v>0.486</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>0.318</v>
+        <v>0.488</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>0.32</v>
+        <v>0.476</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>0.293</v>
+        <v>0.453</v>
       </c>
       <c r="H85" s="36" t="inlineStr">
         <is>
@@ -6252,202 +6134,178 @@
       <c r="I85" s="32" t="inlineStr"/>
       <c r="J85" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="K85" s="32" t="n">
-        <v>0.275</v>
+        <v>0.408</v>
       </c>
       <c r="L85" s="32" t="n">
-        <v>0.281</v>
+        <v>0.441</v>
       </c>
       <c r="M85" s="32" t="n">
-        <v>0.308</v>
+        <v>0.461</v>
       </c>
       <c r="N85" s="32" t="n">
-        <v>0.311</v>
+        <v>0.464</v>
       </c>
       <c r="O85" s="32" t="n">
-        <v>0.342</v>
+        <v>0.481</v>
       </c>
       <c r="P85" s="32" t="n">
-        <v>0.281</v>
+        <v>0.441</v>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.467</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.797</v>
+        <v>0.48</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.822</v>
+        <v>0.486</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.488</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.467</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="H86" s="33" t="inlineStr">
-        <is>
-          <t>4th</t>
+        <v>0.454</v>
+      </c>
+      <c r="H86" s="36" t="inlineStr">
+        <is>
+          <t>12th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
-      <c r="J86" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J86" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K86" s="32" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="L86" s="32" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="M86" s="32" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="N86" s="32" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="O86" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="P86" s="32" t="n">
+        <v>0.449</v>
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>80.69199999999999</v>
+        <v>0.33</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>81.45399999999999</v>
+        <v>0.315</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>81.39700000000001</v>
+        <v>0.318</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>79.672</v>
-      </c>
-      <c r="H87" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
+        <v>0.293</v>
+      </c>
+      <c r="H87" s="36" t="inlineStr">
+        <is>
+          <t>12th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
-      <c r="J87" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J87" s="33" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K87" s="32" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="L87" s="32" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="M87" s="32" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="N87" s="32" t="n">
+        <v>0.311</v>
+      </c>
+      <c r="O87" s="32" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="P87" s="32" t="n">
+        <v>0.281</v>
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>0.543</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>0.54</v>
+        <v>0.797</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>0.54</v>
+        <v>0.822</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>0.547</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>0.543</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>0.519</v>
-      </c>
-      <c r="H88" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>0.821</v>
+      </c>
+      <c r="H88" s="33" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
@@ -6488,37 +6346,37 @@
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>0.225</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>0.228</v>
+        <v>80.69199999999999</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>0.231</v>
+        <v>81.45399999999999</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>0.226</v>
+        <v>81.39700000000001</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>0.225</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>0.231</v>
-      </c>
-      <c r="H89" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
+        <v>79.672</v>
+      </c>
+      <c r="H89" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -6559,96 +6417,108 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>31.2</v>
+        <v>0.543</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>34.167</v>
+        <v>0.54</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>34.5</v>
+        <v>0.54</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>32.867</v>
+        <v>0.547</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>31.2</v>
+        <v>0.543</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>29.6</v>
+        <v>0.519</v>
       </c>
       <c r="H90" s="36" t="inlineStr">
         <is>
-          <t>13th</t>
+          <t>11th</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
-      <c r="J90" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K90" s="32" t="n">
-        <v>30</v>
-      </c>
-      <c r="L90" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="M90" s="32" t="n">
-        <v>33.615</v>
-      </c>
-      <c r="N90" s="32" t="n">
-        <v>33.444</v>
-      </c>
-      <c r="O90" s="32" t="n">
-        <v>32.893</v>
-      </c>
-      <c r="P90" s="32" t="n">
-        <v>32.75</v>
+      <c r="J90" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B91" s="32" t="n">
-        <v>17.7</v>
+        <v>0.225</v>
       </c>
       <c r="C91" s="32" t="n">
-        <v>19.933</v>
+        <v>0.228</v>
       </c>
       <c r="D91" s="32" t="n">
-        <v>18.9</v>
+        <v>0.231</v>
       </c>
       <c r="E91" s="32" t="n">
-        <v>17.867</v>
+        <v>0.226</v>
       </c>
       <c r="F91" s="32" t="n">
-        <v>17.7</v>
+        <v>0.225</v>
       </c>
       <c r="G91" s="32" t="n">
-        <v>16.4</v>
+        <v>0.231</v>
       </c>
       <c r="H91" s="36" t="inlineStr">
         <is>
-          <t>13th</t>
+          <t>10th</t>
         </is>
       </c>
       <c r="I91" s="32" t="inlineStr"/>
@@ -6689,108 +6559,96 @@
       </c>
       <c r="Q91" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B92" s="32" t="n">
-        <v>11.1</v>
+        <v>31.2</v>
       </c>
       <c r="C92" s="32" t="n">
-        <v>10.967</v>
+        <v>34.167</v>
       </c>
       <c r="D92" s="32" t="n">
-        <v>10.15</v>
+        <v>34.5</v>
       </c>
       <c r="E92" s="32" t="n">
-        <v>9.933</v>
+        <v>32.867</v>
       </c>
       <c r="F92" s="32" t="n">
-        <v>11.1</v>
+        <v>31.2</v>
       </c>
       <c r="G92" s="32" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="H92" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
+        <v>29.6</v>
+      </c>
+      <c r="H92" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
         </is>
       </c>
       <c r="I92" s="32" t="inlineStr"/>
-      <c r="J92" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J92" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K92" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="L92" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="M92" s="32" t="n">
+        <v>33.615</v>
+      </c>
+      <c r="N92" s="32" t="n">
+        <v>33.444</v>
+      </c>
+      <c r="O92" s="32" t="n">
+        <v>32.893</v>
+      </c>
+      <c r="P92" s="32" t="n">
+        <v>32.75</v>
       </c>
       <c r="Q92" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B93" s="32" t="n">
-        <v>12.6</v>
+        <v>17.7</v>
       </c>
       <c r="C93" s="32" t="n">
-        <v>12.267</v>
+        <v>19.933</v>
       </c>
       <c r="D93" s="32" t="n">
-        <v>12.5</v>
+        <v>18.9</v>
       </c>
       <c r="E93" s="32" t="n">
-        <v>12.733</v>
+        <v>17.867</v>
       </c>
       <c r="F93" s="32" t="n">
-        <v>12.6</v>
+        <v>17.7</v>
       </c>
       <c r="G93" s="32" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="H93" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
+        <v>16.4</v>
+      </c>
+      <c r="H93" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
         </is>
       </c>
       <c r="I93" s="32" t="inlineStr"/>
@@ -6831,253 +6689,269 @@
       </c>
       <c r="Q93" s="34" t="inlineStr">
         <is>
+          <t>Opp AST</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B94" s="32" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C94" s="32" t="n">
+        <v>10.967</v>
+      </c>
+      <c r="D94" s="32" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="E94" s="32" t="n">
+        <v>9.933</v>
+      </c>
+      <c r="F94" s="32" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="G94" s="32" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H94" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="I94" s="32" t="inlineStr"/>
+      <c r="J94" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q94" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="31" t="inlineStr">
+        <is>
+          <t>TOV</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="C95" s="32" t="n">
+        <v>12.267</v>
+      </c>
+      <c r="D95" s="32" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E95" s="32" t="n">
+        <v>12.733</v>
+      </c>
+      <c r="F95" s="32" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G95" s="32" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="H95" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="inlineStr"/>
+      <c r="J95" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q95" s="34" t="inlineStr">
+        <is>
           <t>Opp TOV</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="29" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="29" t="inlineStr">
         <is>
           <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="30" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B96" s="30" t="inlineStr">
+      <c r="B98" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C96" s="30" t="inlineStr">
+      <c r="C98" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D96" s="30" t="inlineStr">
+      <c r="D98" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E96" s="30" t="inlineStr">
+      <c r="E98" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F96" s="30" t="inlineStr">
+      <c r="F98" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G96" s="30" t="inlineStr">
+      <c r="G98" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H96" s="30" t="inlineStr">
+      <c r="H98" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I96" s="30" t="inlineStr">
+      <c r="I98" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J96" s="30" t="inlineStr">
+      <c r="J98" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K96" s="30" t="inlineStr">
+      <c r="K98" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L96" s="30" t="inlineStr">
+      <c r="L98" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M96" s="30" t="inlineStr">
+      <c r="M98" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N96" s="30" t="inlineStr">
+      <c r="N98" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O96" s="30" t="inlineStr">
+      <c r="O98" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P96" s="30" t="inlineStr">
+      <c r="P98" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q96" s="30" t="inlineStr">
+      <c r="Q98" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="31" t="inlineStr">
-        <is>
-          <t>PPG</t>
-        </is>
-      </c>
-      <c r="B97" s="32" t="n">
-        <v>89.09999999999999</v>
-      </c>
-      <c r="C97" s="32" t="n">
-        <v>85.2</v>
-      </c>
-      <c r="D97" s="32" t="n">
-        <v>84.90000000000001</v>
-      </c>
-      <c r="E97" s="32" t="n">
-        <v>85.867</v>
-      </c>
-      <c r="F97" s="32" t="n">
-        <v>89.09999999999999</v>
-      </c>
-      <c r="G97" s="32" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="H97" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I97" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J97" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K97" s="32" t="n">
-        <v>89.8</v>
-      </c>
-      <c r="L97" s="32" t="n">
-        <v>86.77800000000001</v>
-      </c>
-      <c r="M97" s="32" t="n">
-        <v>87.786</v>
-      </c>
-      <c r="N97" s="32" t="n">
-        <v>84.36799999999999</v>
-      </c>
-      <c r="O97" s="32" t="n">
-        <v>82.655</v>
-      </c>
-      <c r="P97" s="32" t="n">
-        <v>86.77800000000001</v>
-      </c>
-      <c r="Q97" s="34" t="inlineStr">
-        <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B98" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="C98" s="32" t="n">
-        <v>107.942</v>
-      </c>
-      <c r="D98" s="32" t="n">
-        <v>105.587</v>
-      </c>
-      <c r="E98" s="32" t="n">
-        <v>105.509</v>
-      </c>
-      <c r="F98" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="G98" s="32" t="n">
-        <v>115.565</v>
-      </c>
-      <c r="H98" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I98" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J98" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K98" s="32" t="n">
-        <v>113.552</v>
-      </c>
-      <c r="L98" s="32" t="n">
-        <v>108.265</v>
-      </c>
-      <c r="M98" s="32" t="n">
-        <v>109.197</v>
-      </c>
-      <c r="N98" s="32" t="n">
-        <v>104.078</v>
-      </c>
-      <c r="O98" s="32" t="n">
-        <v>102.45</v>
-      </c>
-      <c r="P98" s="32" t="n">
-        <v>108.265</v>
-      </c>
-      <c r="Q98" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>0.544</v>
+        <v>85.2</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>0.533</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>0.535</v>
+        <v>85.867</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>0.579</v>
+        <v>94.2</v>
       </c>
       <c r="H99" s="33" t="inlineStr">
         <is>
@@ -7095,52 +6969,52 @@
         </is>
       </c>
       <c r="K99" s="32" t="n">
-        <v>0.571</v>
+        <v>89.8</v>
       </c>
       <c r="L99" s="32" t="n">
-        <v>0.545</v>
+        <v>86.77800000000001</v>
       </c>
       <c r="M99" s="32" t="n">
-        <v>0.53</v>
+        <v>87.786</v>
       </c>
       <c r="N99" s="32" t="n">
-        <v>0.506</v>
+        <v>84.36799999999999</v>
       </c>
       <c r="O99" s="32" t="n">
-        <v>0.5</v>
+        <v>82.655</v>
       </c>
       <c r="P99" s="32" t="n">
-        <v>0.545</v>
+        <v>86.77800000000001</v>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>109.659</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>0.534</v>
+        <v>107.942</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>0.543</v>
+        <v>105.587</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>0.549</v>
+        <v>105.509</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>109.659</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>0.582</v>
+        <v>115.565</v>
       </c>
       <c r="H100" s="33" t="inlineStr">
         <is>
@@ -7149,65 +7023,65 @@
       </c>
       <c r="I100" s="32" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="J100" s="36" t="inlineStr">
         <is>
-          <t>10th</t>
+          <t>14th</t>
         </is>
       </c>
       <c r="K100" s="32" t="n">
-        <v>0.5</v>
+        <v>113.552</v>
       </c>
       <c r="L100" s="32" t="n">
-        <v>0.514</v>
+        <v>108.265</v>
       </c>
       <c r="M100" s="32" t="n">
-        <v>0.5</v>
+        <v>109.197</v>
       </c>
       <c r="N100" s="32" t="n">
-        <v>0.494</v>
+        <v>104.078</v>
       </c>
       <c r="O100" s="32" t="n">
-        <v>0.497</v>
+        <v>102.45</v>
       </c>
       <c r="P100" s="32" t="n">
-        <v>0.514</v>
+        <v>108.265</v>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>0.373</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>0.374</v>
+        <v>0.544</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>0.343</v>
+        <v>0.533</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>0.347</v>
+        <v>0.535</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>0.373</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>0.382</v>
+        <v>0.579</v>
       </c>
       <c r="H101" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I101" s="32" t="inlineStr">
@@ -7221,198 +7095,182 @@
         </is>
       </c>
       <c r="K101" s="32" t="n">
-        <v>0.453</v>
+        <v>0.571</v>
       </c>
       <c r="L101" s="32" t="n">
-        <v>0.39</v>
+        <v>0.545</v>
       </c>
       <c r="M101" s="32" t="n">
-        <v>0.381</v>
+        <v>0.53</v>
       </c>
       <c r="N101" s="32" t="n">
-        <v>0.347</v>
+        <v>0.506</v>
       </c>
       <c r="O101" s="32" t="n">
-        <v>0.337</v>
+        <v>0.5</v>
       </c>
       <c r="P101" s="32" t="n">
-        <v>0.39</v>
+        <v>0.545</v>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
-        <v>0.767</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="C102" s="32" t="n">
-        <v>0.744</v>
+        <v>0.534</v>
       </c>
       <c r="D102" s="32" t="n">
-        <v>0.749</v>
+        <v>0.543</v>
       </c>
       <c r="E102" s="32" t="n">
-        <v>0.779</v>
+        <v>0.549</v>
       </c>
       <c r="F102" s="32" t="n">
-        <v>0.767</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="G102" s="32" t="n">
-        <v>0.842</v>
+        <v>0.582</v>
       </c>
       <c r="H102" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="I102" s="32" t="inlineStr"/>
-      <c r="J102" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I102" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J102" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K102" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L102" s="32" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="M102" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N102" s="32" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="O102" s="32" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="P102" s="32" t="n">
+        <v>0.514</v>
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>81.724</v>
+        <v>0.373</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>79.247</v>
+        <v>0.374</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>80.62</v>
+        <v>0.343</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>81.736</v>
+        <v>0.347</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>81.724</v>
+        <v>0.373</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>82.304</v>
-      </c>
-      <c r="H103" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I103" s="32" t="inlineStr"/>
-      <c r="J103" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.382</v>
+      </c>
+      <c r="H103" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I103" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J103" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K103" s="32" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="L103" s="32" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="M103" s="32" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="N103" s="32" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="O103" s="32" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="P103" s="32" t="n">
+        <v>0.39</v>
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>0.591</v>
+        <v>0.767</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>0.57</v>
+        <v>0.744</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.749</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.779</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>0.591</v>
+        <v>0.767</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>0.613</v>
+        <v>0.842</v>
       </c>
       <c r="H104" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="I104" s="32" t="inlineStr"/>
@@ -7453,37 +7311,37 @@
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>0.265</v>
+        <v>81.724</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>0.255</v>
+        <v>79.247</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>0.253</v>
+        <v>80.62</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>0.245</v>
+        <v>81.736</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>0.265</v>
+        <v>81.724</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>0.287</v>
-      </c>
-      <c r="H105" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
+        <v>82.304</v>
+      </c>
+      <c r="H105" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -7524,100 +7382,108 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>37.6</v>
+        <v>0.591</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>34.9</v>
+        <v>0.57</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>36.05</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>36.467</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>37.6</v>
+        <v>0.591</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>40.4</v>
+        <v>0.613</v>
       </c>
       <c r="H106" s="33" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I106" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J106" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K106" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="L106" s="32" t="n">
-        <v>34.556</v>
-      </c>
-      <c r="M106" s="32" t="n">
-        <v>34.929</v>
-      </c>
-      <c r="N106" s="32" t="n">
-        <v>35.053</v>
-      </c>
-      <c r="O106" s="32" t="n">
-        <v>35.69</v>
-      </c>
-      <c r="P106" s="32" t="n">
-        <v>34.556</v>
+      <c r="I106" s="32" t="inlineStr"/>
+      <c r="J106" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q106" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B107" s="32" t="n">
-        <v>21.1</v>
+        <v>0.265</v>
       </c>
       <c r="C107" s="32" t="n">
-        <v>21.533</v>
+        <v>0.255</v>
       </c>
       <c r="D107" s="32" t="n">
-        <v>21.1</v>
+        <v>0.253</v>
       </c>
       <c r="E107" s="32" t="n">
-        <v>20.867</v>
+        <v>0.245</v>
       </c>
       <c r="F107" s="32" t="n">
-        <v>21.1</v>
+        <v>0.265</v>
       </c>
       <c r="G107" s="32" t="n">
-        <v>23.2</v>
+        <v>0.287</v>
       </c>
       <c r="H107" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I107" s="32" t="inlineStr"/>
@@ -7658,108 +7524,100 @@
       </c>
       <c r="Q107" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B108" s="32" t="n">
-        <v>13</v>
+        <v>37.6</v>
       </c>
       <c r="C108" s="32" t="n">
-        <v>12.567</v>
+        <v>34.9</v>
       </c>
       <c r="D108" s="32" t="n">
-        <v>13.05</v>
+        <v>36.05</v>
       </c>
       <c r="E108" s="32" t="n">
-        <v>12.867</v>
+        <v>36.467</v>
       </c>
       <c r="F108" s="32" t="n">
-        <v>13</v>
+        <v>37.6</v>
       </c>
       <c r="G108" s="32" t="n">
-        <v>14.2</v>
+        <v>40.4</v>
       </c>
       <c r="H108" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I108" s="32" t="inlineStr"/>
-      <c r="J108" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I108" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J108" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K108" s="32" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="L108" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="M108" s="32" t="n">
+        <v>34.929</v>
+      </c>
+      <c r="N108" s="32" t="n">
+        <v>35.053</v>
+      </c>
+      <c r="O108" s="32" t="n">
+        <v>35.69</v>
+      </c>
+      <c r="P108" s="32" t="n">
+        <v>34.556</v>
       </c>
       <c r="Q108" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B109" s="32" t="n">
-        <v>14.8</v>
+        <v>21.1</v>
       </c>
       <c r="C109" s="32" t="n">
-        <v>12.733</v>
+        <v>21.533</v>
       </c>
       <c r="D109" s="32" t="n">
-        <v>13.35</v>
+        <v>21.1</v>
       </c>
       <c r="E109" s="32" t="n">
-        <v>13.733</v>
+        <v>20.867</v>
       </c>
       <c r="F109" s="32" t="n">
-        <v>14.8</v>
+        <v>21.1</v>
       </c>
       <c r="G109" s="32" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H109" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>23.2</v>
+      </c>
+      <c r="H109" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="I109" s="32" t="inlineStr"/>
@@ -7799,6 +7657,148 @@
         </is>
       </c>
       <c r="Q109" s="34" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C110" s="32" t="n">
+        <v>12.567</v>
+      </c>
+      <c r="D110" s="32" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="E110" s="32" t="n">
+        <v>12.867</v>
+      </c>
+      <c r="F110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="G110" s="32" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H110" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I110" s="32" t="inlineStr"/>
+      <c r="J110" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q110" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="31" t="inlineStr">
+        <is>
+          <t>TOV</t>
+        </is>
+      </c>
+      <c r="B111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C111" s="32" t="n">
+        <v>12.733</v>
+      </c>
+      <c r="D111" s="32" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="E111" s="32" t="n">
+        <v>13.733</v>
+      </c>
+      <c r="F111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="G111" s="32" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H111" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I111" s="32" t="inlineStr"/>
+      <c r="J111" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q111" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>

</xml_diff>

<commit_message>
data: hourly update 2026-07-13 15:46Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-13.xlsx
+++ b/data/output/workbook/2026-07-13.xlsx
@@ -363,7 +363,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12877800"/>
+    <ext cx="10125075" cy="12306300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 04:21</t>
+          <t>2026-07-13 11:46</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1128,14 +1128,14 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.604</v>
+        <v>0.617</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-153</v>
+        <v>-161</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>-108</v>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 60.4% (fair -153). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1189,22 +1189,22 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5438</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-119</v>
+        <v>-125</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1255,22 +1255,22 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 171.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5429</v>
+        <v>0.5438</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>-119</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1330,13 +1330,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5574</v>
+        <v>0.5575</v>
       </c>
       <c r="G8" s="14" t="n">
         <v>-126</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 55.7% (fair -126). Your call.</t>
+          <t>Model 55.8% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1369,75 +1369,9 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury @ Minnesota Lynx</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>01:00</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Over 169.5</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>0.5187</v>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>-108</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>-102</v>
-      </c>
-      <c r="I9" s="13">
-        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
-        <v/>
-      </c>
-      <c r="J9" s="16">
-        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
-        <v/>
-      </c>
-      <c r="K9" s="17">
-        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L9" s="18">
-        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M9" s="12">
-        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N9" s="19" t="inlineStr">
-        <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
-        </is>
-      </c>
-      <c r="O9" s="15" t="n"/>
-      <c r="P9" s="16">
-        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J9">
+  <conditionalFormatting sqref="J5:J8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1944,7 +1878,7 @@
         <v>-202</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-120</v>
+        <v>-115</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -2000,17 +1934,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 180.5</t>
+          <t>Over 182.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5316474443436277</v>
+        <v>0.4847500404119037</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-114</v>
+        <v>106</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -2034,7 +1968,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -2066,17 +2000,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 180.5</t>
+          <t>Under 182.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4683525556563723</v>
+        <v>0.5152499595880963</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>114</v>
+        <v>-106</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2100,7 +2034,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2132,17 +2066,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream -8.5</t>
+          <t>Atlanta Dream -9.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4210482224080958</v>
+        <v>0.3905243127429648</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2166,7 +2100,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 42.1% (fair +138). Your call.</t>
+          <t>Model 39.1% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -2198,17 +2132,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks +8.5</t>
+          <t>Los Angeles Sparks +9.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5789517775919042</v>
+        <v>0.6094756872570352</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-138</v>
+        <v>-156</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2232,7 +2166,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 57.9% (fair -138). Your call.</t>
+          <t>Model 60.9% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -2396,17 +2330,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 169.5</t>
+          <t>Over 170</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5187</v>
+        <v>0.5063</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-108</v>
+        <v>-103</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-102</v>
+        <v>-101</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2430,7 +2364,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 50.6% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2462,14 +2396,14 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 169.5</t>
+          <t>Under 170</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4813</v>
+        <v>0.4703000000000001</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>104</v>
@@ -2496,7 +2430,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2528,17 +2462,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Lynx -13.5</t>
+          <t>Minnesota Lynx -12.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.46486323937778</v>
+        <v>0.4962305227318936</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -2562,7 +2496,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -2594,17 +2528,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury +13.5</t>
+          <t>Phoenix Mercury +12.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.53513676062222</v>
+        <v>0.5037694772681064</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-115</v>
+        <v>-102</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -2628,7 +2562,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -2664,13 +2598,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4426</v>
+        <v>0.4425</v>
       </c>
       <c r="G17" s="14" t="n">
         <v>126</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -2694,7 +2628,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 44.3% (fair +126). Your call.</t>
+          <t>Model 44.2% (fair +126). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -2730,13 +2664,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5574</v>
+        <v>0.5575</v>
       </c>
       <c r="G18" s="14" t="n">
         <v>-126</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -2760,7 +2694,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 55.7% (fair -126). Your call.</t>
+          <t>Model 55.8% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -2792,14 +2726,14 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.604</v>
+        <v>0.617</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-153</v>
+        <v>-161</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>-108</v>
@@ -2826,7 +2760,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 60.4% (fair -153). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2858,17 +2792,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 168.5</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.396</v>
+        <v>0.383</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -2892,7 +2826,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 39.6% (fair +153). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -2928,13 +2862,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4965</v>
+        <v>0.4930895344612759</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -2958,7 +2892,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +101). Your call.</t>
+          <t>Model 49.3% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -2994,13 +2928,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5035000000000001</v>
+        <v>0.5069104655387241</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-101</v>
+        <v>-103</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -3024,7 +2958,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -101). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -3188,17 +3122,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 171.5</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5429</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-119</v>
+        <v>-125</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -3222,7 +3156,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -3254,17 +3188,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 171.5</t>
+          <t>Under 170.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4571</v>
+        <v>0.4441000000000001</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -3288,7 +3222,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -3324,13 +3258,13 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5057</v>
+        <v>0.5053400127859651</v>
       </c>
       <c r="G27" s="14" t="n">
         <v>-102</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -3354,7 +3288,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -102). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -3390,13 +3324,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4943</v>
+        <v>0.4946599872140349</v>
       </c>
       <c r="G28" s="14" t="n">
         <v>102</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -3420,7 +3354,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +102). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -5873,7 +5807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q111"/>
+  <dimension ref="A1:Q107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5890,493 +5824,765 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B78" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C78" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D78" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E78" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F78" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G78" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H78" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I78" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J78" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K78" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L78" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M78" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N78" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O78" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P78" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q78" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="31" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="B79" s="32" t="n">
+        <v>83</v>
+      </c>
+      <c r="C79" s="32" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="D79" s="32" t="n">
+        <v>83.05</v>
+      </c>
+      <c r="E79" s="32" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="F79" s="32" t="n">
+        <v>83</v>
+      </c>
+      <c r="G79" s="32" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="H79" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I79" s="32" t="inlineStr"/>
+      <c r="J79" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="n">
+        <v>72.75</v>
+      </c>
+      <c r="L79" s="32" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="M79" s="32" t="n">
+        <v>80</v>
+      </c>
+      <c r="N79" s="32" t="n">
+        <v>78.72199999999999</v>
+      </c>
+      <c r="O79" s="32" t="n">
+        <v>79</v>
+      </c>
+      <c r="P79" s="32" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="Q79" s="34" t="inlineStr">
+        <is>
+          <t>Opp PPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B80" s="32" t="n">
+        <v>101.929</v>
+      </c>
+      <c r="C80" s="32" t="n">
+        <v>102.13</v>
+      </c>
+      <c r="D80" s="32" t="n">
+        <v>101.973</v>
+      </c>
+      <c r="E80" s="32" t="n">
+        <v>102.639</v>
+      </c>
+      <c r="F80" s="32" t="n">
+        <v>101.929</v>
+      </c>
+      <c r="G80" s="32" t="n">
+        <v>97.006</v>
+      </c>
+      <c r="H80" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr"/>
+      <c r="J80" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K80" s="32" t="n">
+        <v>88.01600000000001</v>
+      </c>
+      <c r="L80" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="M80" s="32" t="n">
+        <v>97.129</v>
+      </c>
+      <c r="N80" s="32" t="n">
+        <v>96.706</v>
+      </c>
+      <c r="O80" s="32" t="n">
+        <v>98.628</v>
+      </c>
+      <c r="P80" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="Q80" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
+        </is>
+      </c>
+    </row>
     <row r="81">
-      <c r="A81" s="29" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
+      <c r="A81" s="31" t="inlineStr">
+        <is>
+          <t>eFG%</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>0.476</v>
+      </c>
+      <c r="C81" s="32" t="n">
+        <v>0.491</v>
+      </c>
+      <c r="D81" s="32" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="E81" s="32" t="n">
+        <v>0.488</v>
+      </c>
+      <c r="F81" s="32" t="n">
+        <v>0.476</v>
+      </c>
+      <c r="G81" s="32" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="H81" s="36" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr"/>
+      <c r="J81" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="L81" s="32" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="M81" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="N81" s="32" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="O81" s="32" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="P81" s="32" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="Q81" s="34" t="inlineStr">
+        <is>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B82" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C82" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D82" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E82" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F82" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G82" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H82" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I82" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J82" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K82" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L82" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M82" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N82" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O82" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P82" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q82" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A82" s="31" t="inlineStr">
+        <is>
+          <t>2PT%</t>
+        </is>
+      </c>
+      <c r="B82" s="32" t="n">
+        <v>0.467</v>
+      </c>
+      <c r="C82" s="32" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D82" s="32" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="E82" s="32" t="n">
+        <v>0.488</v>
+      </c>
+      <c r="F82" s="32" t="n">
+        <v>0.467</v>
+      </c>
+      <c r="G82" s="32" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="H82" s="36" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="inlineStr"/>
+      <c r="J82" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K82" s="32" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="L82" s="32" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="M82" s="32" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="N82" s="32" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="O82" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="P82" s="32" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="Q82" s="34" t="inlineStr">
+        <is>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>83</v>
+        <v>0.32</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>82.3</v>
+        <v>0.33</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>83.05</v>
+        <v>0.315</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>83.59999999999999</v>
+        <v>0.318</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>83</v>
+        <v>0.32</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>77.40000000000001</v>
+        <v>0.293</v>
       </c>
       <c r="H83" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I83" s="32" t="inlineStr"/>
       <c r="J83" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="K83" s="32" t="n">
-        <v>72.75</v>
+        <v>0.275</v>
       </c>
       <c r="L83" s="32" t="n">
-        <v>79.75</v>
+        <v>0.281</v>
       </c>
       <c r="M83" s="32" t="n">
-        <v>80</v>
+        <v>0.308</v>
       </c>
       <c r="N83" s="32" t="n">
-        <v>78.72199999999999</v>
+        <v>0.311</v>
       </c>
       <c r="O83" s="32" t="n">
-        <v>79</v>
+        <v>0.342</v>
       </c>
       <c r="P83" s="32" t="n">
-        <v>79.75</v>
+        <v>0.281</v>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>101.929</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>102.13</v>
+        <v>0.797</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>101.973</v>
+        <v>0.822</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>102.639</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>101.929</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>97.006</v>
-      </c>
-      <c r="H84" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>0.821</v>
+      </c>
+      <c r="H84" s="33" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
-      <c r="J84" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K84" s="32" t="n">
-        <v>88.01600000000001</v>
-      </c>
-      <c r="L84" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="M84" s="32" t="n">
-        <v>97.129</v>
-      </c>
-      <c r="N84" s="32" t="n">
-        <v>96.706</v>
-      </c>
-      <c r="O84" s="32" t="n">
-        <v>98.628</v>
-      </c>
-      <c r="P84" s="32" t="n">
-        <v>95.66500000000001</v>
+      <c r="J84" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>0.476</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>0.491</v>
+        <v>80.69199999999999</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>0.486</v>
+        <v>81.45399999999999</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>0.488</v>
+        <v>81.39700000000001</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>0.476</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>0.453</v>
-      </c>
-      <c r="H85" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
+        <v>79.672</v>
+      </c>
+      <c r="H85" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
         </is>
       </c>
       <c r="I85" s="32" t="inlineStr"/>
-      <c r="J85" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K85" s="32" t="n">
-        <v>0.408</v>
-      </c>
-      <c r="L85" s="32" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="M85" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="N85" s="32" t="n">
-        <v>0.464</v>
-      </c>
-      <c r="O85" s="32" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="P85" s="32" t="n">
-        <v>0.441</v>
+      <c r="J85" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.467</v>
+        <v>0.543</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.48</v>
+        <v>0.54</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.486</v>
+        <v>0.54</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.488</v>
+        <v>0.547</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.467</v>
+        <v>0.543</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.454</v>
+        <v>0.519</v>
       </c>
       <c r="H86" s="36" t="inlineStr">
         <is>
-          <t>12th</t>
+          <t>11th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
-      <c r="J86" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K86" s="32" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="L86" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="M86" s="32" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="N86" s="32" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="O86" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="P86" s="32" t="n">
-        <v>0.449</v>
+      <c r="J86" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>0.32</v>
+        <v>0.225</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>0.33</v>
+        <v>0.228</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>0.315</v>
+        <v>0.231</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>0.318</v>
+        <v>0.226</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>0.32</v>
+        <v>0.225</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>0.293</v>
+        <v>0.231</v>
       </c>
       <c r="H87" s="36" t="inlineStr">
         <is>
-          <t>12th</t>
+          <t>10th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
-      <c r="J87" s="33" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="K87" s="32" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="L87" s="32" t="n">
-        <v>0.281</v>
-      </c>
-      <c r="M87" s="32" t="n">
-        <v>0.308</v>
-      </c>
-      <c r="N87" s="32" t="n">
-        <v>0.311</v>
-      </c>
-      <c r="O87" s="32" t="n">
-        <v>0.342</v>
-      </c>
-      <c r="P87" s="32" t="n">
-        <v>0.281</v>
+      <c r="J87" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>31.2</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>0.797</v>
+        <v>34.167</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>0.822</v>
+        <v>34.5</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>0.8070000000000001</v>
+        <v>32.867</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>31.2</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="H88" s="33" t="inlineStr">
-        <is>
-          <t>4th</t>
+        <v>29.6</v>
+      </c>
+      <c r="H88" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
-      <c r="J88" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J88" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K88" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="L88" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="M88" s="32" t="n">
+        <v>33.615</v>
+      </c>
+      <c r="N88" s="32" t="n">
+        <v>33.444</v>
+      </c>
+      <c r="O88" s="32" t="n">
+        <v>32.893</v>
+      </c>
+      <c r="P88" s="32" t="n">
+        <v>32.75</v>
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>17.7</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>80.69199999999999</v>
+        <v>19.933</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>81.45399999999999</v>
+        <v>18.9</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>81.39700000000001</v>
+        <v>17.867</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>17.7</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>79.672</v>
-      </c>
-      <c r="H89" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
+        <v>16.4</v>
+      </c>
+      <c r="H89" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -6417,37 +6623,37 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>0.543</v>
+        <v>11.1</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>0.54</v>
+        <v>10.967</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>0.54</v>
+        <v>10.15</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>0.547</v>
+        <v>9.933</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>0.543</v>
+        <v>11.1</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>0.519</v>
-      </c>
-      <c r="H90" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>11.4</v>
+      </c>
+      <c r="H90" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
@@ -6488,37 +6694,37 @@
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B91" s="32" t="n">
-        <v>0.225</v>
+        <v>12.6</v>
       </c>
       <c r="C91" s="32" t="n">
-        <v>0.228</v>
+        <v>12.267</v>
       </c>
       <c r="D91" s="32" t="n">
-        <v>0.231</v>
+        <v>12.5</v>
       </c>
       <c r="E91" s="32" t="n">
-        <v>0.226</v>
+        <v>12.733</v>
       </c>
       <c r="F91" s="32" t="n">
-        <v>0.225</v>
+        <v>12.6</v>
       </c>
       <c r="G91" s="32" t="n">
-        <v>0.231</v>
-      </c>
-      <c r="H91" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
+        <v>13.4</v>
+      </c>
+      <c r="H91" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I91" s="32" t="inlineStr"/>
@@ -6559,403 +6765,383 @@
       </c>
       <c r="Q91" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="31" t="inlineStr">
-        <is>
-          <t>REB</t>
-        </is>
-      </c>
-      <c r="B92" s="32" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="C92" s="32" t="n">
-        <v>34.167</v>
-      </c>
-      <c r="D92" s="32" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="E92" s="32" t="n">
-        <v>32.867</v>
-      </c>
-      <c r="F92" s="32" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="G92" s="32" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="H92" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
-        </is>
-      </c>
-      <c r="I92" s="32" t="inlineStr"/>
-      <c r="J92" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K92" s="32" t="n">
-        <v>30</v>
-      </c>
-      <c r="L92" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="M92" s="32" t="n">
-        <v>33.615</v>
-      </c>
-      <c r="N92" s="32" t="n">
-        <v>33.444</v>
-      </c>
-      <c r="O92" s="32" t="n">
-        <v>32.893</v>
-      </c>
-      <c r="P92" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="Q92" s="34" t="inlineStr">
-        <is>
-          <t>Opp REB</t>
+          <t>Opp TOV</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="31" t="inlineStr">
-        <is>
-          <t>AST</t>
-        </is>
-      </c>
-      <c r="B93" s="32" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="C93" s="32" t="n">
-        <v>19.933</v>
-      </c>
-      <c r="D93" s="32" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="E93" s="32" t="n">
-        <v>17.867</v>
-      </c>
-      <c r="F93" s="32" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G93" s="32" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="H93" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
-        </is>
-      </c>
-      <c r="I93" s="32" t="inlineStr"/>
-      <c r="J93" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q93" s="34" t="inlineStr">
-        <is>
-          <t>Opp AST</t>
+      <c r="A93" s="29" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B94" s="32" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="C94" s="32" t="n">
-        <v>10.967</v>
-      </c>
-      <c r="D94" s="32" t="n">
-        <v>10.15</v>
-      </c>
-      <c r="E94" s="32" t="n">
-        <v>9.933</v>
-      </c>
-      <c r="F94" s="32" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="G94" s="32" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="H94" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="I94" s="32" t="inlineStr"/>
-      <c r="J94" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q94" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
+      <c r="A94" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B94" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C94" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D94" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F94" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G94" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H94" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I94" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J94" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K94" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L94" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M94" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N94" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O94" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P94" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q94" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B95" s="32" t="n">
-        <v>12.6</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="C95" s="32" t="n">
-        <v>12.267</v>
+        <v>85.2</v>
       </c>
       <c r="D95" s="32" t="n">
-        <v>12.5</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E95" s="32" t="n">
-        <v>12.733</v>
+        <v>85.867</v>
       </c>
       <c r="F95" s="32" t="n">
-        <v>12.6</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G95" s="32" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="H95" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I95" s="32" t="inlineStr"/>
-      <c r="J95" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>94.2</v>
+      </c>
+      <c r="H95" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J95" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K95" s="32" t="n">
+        <v>89.8</v>
+      </c>
+      <c r="L95" s="32" t="n">
+        <v>86.77800000000001</v>
+      </c>
+      <c r="M95" s="32" t="n">
+        <v>87.786</v>
+      </c>
+      <c r="N95" s="32" t="n">
+        <v>84.36799999999999</v>
+      </c>
+      <c r="O95" s="32" t="n">
+        <v>82.655</v>
+      </c>
+      <c r="P95" s="32" t="n">
+        <v>86.77800000000001</v>
       </c>
       <c r="Q95" s="34" t="inlineStr">
         <is>
-          <t>Opp TOV</t>
+          <t>Opp PPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B96" s="32" t="n">
+        <v>109.659</v>
+      </c>
+      <c r="C96" s="32" t="n">
+        <v>107.942</v>
+      </c>
+      <c r="D96" s="32" t="n">
+        <v>105.587</v>
+      </c>
+      <c r="E96" s="32" t="n">
+        <v>105.509</v>
+      </c>
+      <c r="F96" s="32" t="n">
+        <v>109.659</v>
+      </c>
+      <c r="G96" s="32" t="n">
+        <v>115.565</v>
+      </c>
+      <c r="H96" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I96" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J96" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K96" s="32" t="n">
+        <v>113.552</v>
+      </c>
+      <c r="L96" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="M96" s="32" t="n">
+        <v>109.197</v>
+      </c>
+      <c r="N96" s="32" t="n">
+        <v>104.078</v>
+      </c>
+      <c r="O96" s="32" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="P96" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="Q96" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="29" t="inlineStr">
-        <is>
-          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
+      <c r="A97" s="31" t="inlineStr">
+        <is>
+          <t>eFG%</t>
+        </is>
+      </c>
+      <c r="B97" s="32" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="C97" s="32" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="D97" s="32" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="E97" s="32" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="F97" s="32" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="G97" s="32" t="n">
+        <v>0.579</v>
+      </c>
+      <c r="H97" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I97" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J97" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K97" s="32" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="L97" s="32" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="M97" s="32" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N97" s="32" t="n">
+        <v>0.506</v>
+      </c>
+      <c r="O97" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P97" s="32" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="Q97" s="34" t="inlineStr">
+        <is>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B98" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C98" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D98" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E98" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F98" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G98" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H98" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I98" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J98" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K98" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L98" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M98" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N98" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O98" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P98" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q98" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A98" s="31" t="inlineStr">
+        <is>
+          <t>2PT%</t>
+        </is>
+      </c>
+      <c r="B98" s="32" t="n">
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="C98" s="32" t="n">
+        <v>0.534</v>
+      </c>
+      <c r="D98" s="32" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E98" s="32" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="F98" s="32" t="n">
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="G98" s="32" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="H98" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I98" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J98" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K98" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L98" s="32" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="M98" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N98" s="32" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="O98" s="32" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="P98" s="32" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="Q98" s="34" t="inlineStr">
+        <is>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>0.373</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>85.2</v>
+        <v>0.374</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>84.90000000000001</v>
+        <v>0.343</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>85.867</v>
+        <v>0.347</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>0.373</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>94.2</v>
+        <v>0.382</v>
       </c>
       <c r="H99" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I99" s="32" t="inlineStr">
@@ -6969,379 +7155,403 @@
         </is>
       </c>
       <c r="K99" s="32" t="n">
-        <v>89.8</v>
+        <v>0.453</v>
       </c>
       <c r="L99" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>0.39</v>
       </c>
       <c r="M99" s="32" t="n">
-        <v>87.786</v>
+        <v>0.381</v>
       </c>
       <c r="N99" s="32" t="n">
-        <v>84.36799999999999</v>
+        <v>0.347</v>
       </c>
       <c r="O99" s="32" t="n">
-        <v>82.655</v>
+        <v>0.337</v>
       </c>
       <c r="P99" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>0.39</v>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>109.659</v>
+        <v>0.767</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>107.942</v>
+        <v>0.744</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>105.587</v>
+        <v>0.749</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>105.509</v>
+        <v>0.779</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>109.659</v>
+        <v>0.767</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>115.565</v>
+        <v>0.842</v>
       </c>
       <c r="H100" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I100" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J100" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K100" s="32" t="n">
-        <v>113.552</v>
-      </c>
-      <c r="L100" s="32" t="n">
-        <v>108.265</v>
-      </c>
-      <c r="M100" s="32" t="n">
-        <v>109.197</v>
-      </c>
-      <c r="N100" s="32" t="n">
-        <v>104.078</v>
-      </c>
-      <c r="O100" s="32" t="n">
-        <v>102.45</v>
-      </c>
-      <c r="P100" s="32" t="n">
-        <v>108.265</v>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I100" s="32" t="inlineStr"/>
+      <c r="J100" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>81.724</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>0.544</v>
+        <v>79.247</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>0.533</v>
+        <v>80.62</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>0.535</v>
+        <v>81.736</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>81.724</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>0.579</v>
-      </c>
-      <c r="H101" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I101" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J101" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K101" s="32" t="n">
-        <v>0.571</v>
-      </c>
-      <c r="L101" s="32" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="M101" s="32" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N101" s="32" t="n">
-        <v>0.506</v>
-      </c>
-      <c r="O101" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P101" s="32" t="n">
-        <v>0.545</v>
+        <v>82.304</v>
+      </c>
+      <c r="H101" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I101" s="32" t="inlineStr"/>
+      <c r="J101" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
+        <v>0.591</v>
+      </c>
+      <c r="C102" s="32" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="D102" s="32" t="n">
         <v>0.5610000000000001</v>
       </c>
-      <c r="C102" s="32" t="n">
-        <v>0.534</v>
-      </c>
-      <c r="D102" s="32" t="n">
-        <v>0.543</v>
-      </c>
       <c r="E102" s="32" t="n">
-        <v>0.549</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F102" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.591</v>
       </c>
       <c r="G102" s="32" t="n">
-        <v>0.582</v>
+        <v>0.613</v>
       </c>
       <c r="H102" s="33" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I102" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J102" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K102" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L102" s="32" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="M102" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N102" s="32" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="O102" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="P102" s="32" t="n">
-        <v>0.514</v>
+      <c r="I102" s="32" t="inlineStr"/>
+      <c r="J102" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>0.373</v>
+        <v>0.265</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>0.374</v>
+        <v>0.255</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>0.343</v>
+        <v>0.253</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>0.347</v>
+        <v>0.245</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>0.373</v>
+        <v>0.265</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>0.382</v>
+        <v>0.287</v>
       </c>
       <c r="H103" s="33" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="I103" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J103" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K103" s="32" t="n">
-        <v>0.453</v>
-      </c>
-      <c r="L103" s="32" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="M103" s="32" t="n">
-        <v>0.381</v>
-      </c>
-      <c r="N103" s="32" t="n">
-        <v>0.347</v>
-      </c>
-      <c r="O103" s="32" t="n">
-        <v>0.337</v>
-      </c>
-      <c r="P103" s="32" t="n">
-        <v>0.39</v>
+      <c r="I103" s="32" t="inlineStr"/>
+      <c r="J103" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>0.767</v>
+        <v>37.6</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>0.744</v>
+        <v>34.9</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>0.749</v>
+        <v>36.05</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>0.779</v>
+        <v>36.467</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>0.767</v>
+        <v>37.6</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>0.842</v>
+        <v>40.4</v>
       </c>
       <c r="H104" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="I104" s="32" t="inlineStr"/>
-      <c r="J104" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I104" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J104" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K104" s="32" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="L104" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="M104" s="32" t="n">
+        <v>34.929</v>
+      </c>
+      <c r="N104" s="32" t="n">
+        <v>35.053</v>
+      </c>
+      <c r="O104" s="32" t="n">
+        <v>35.69</v>
+      </c>
+      <c r="P104" s="32" t="n">
+        <v>34.556</v>
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>81.724</v>
+        <v>21.1</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>79.247</v>
+        <v>21.533</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>80.62</v>
+        <v>21.1</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>81.736</v>
+        <v>20.867</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>81.724</v>
+        <v>21.1</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>82.304</v>
-      </c>
-      <c r="H105" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
+        <v>23.2</v>
+      </c>
+      <c r="H105" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -7382,37 +7592,37 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>0.591</v>
+        <v>13</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>0.57</v>
+        <v>12.567</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>13.05</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>0.5649999999999999</v>
+        <v>12.867</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>0.591</v>
+        <v>13</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>0.613</v>
+        <v>14.2</v>
       </c>
       <c r="H106" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I106" s="32" t="inlineStr"/>
@@ -7453,37 +7663,37 @@
       </c>
       <c r="Q106" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B107" s="32" t="n">
-        <v>0.265</v>
+        <v>14.8</v>
       </c>
       <c r="C107" s="32" t="n">
-        <v>0.255</v>
+        <v>12.733</v>
       </c>
       <c r="D107" s="32" t="n">
-        <v>0.253</v>
+        <v>13.35</v>
       </c>
       <c r="E107" s="32" t="n">
-        <v>0.245</v>
+        <v>13.733</v>
       </c>
       <c r="F107" s="32" t="n">
-        <v>0.265</v>
+        <v>14.8</v>
       </c>
       <c r="G107" s="32" t="n">
-        <v>0.287</v>
-      </c>
-      <c r="H107" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
+        <v>14.4</v>
+      </c>
+      <c r="H107" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
         </is>
       </c>
       <c r="I107" s="32" t="inlineStr"/>
@@ -7523,282 +7733,6 @@
         </is>
       </c>
       <c r="Q107" s="34" t="inlineStr">
-        <is>
-          <t>Opp OREB%</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="31" t="inlineStr">
-        <is>
-          <t>REB</t>
-        </is>
-      </c>
-      <c r="B108" s="32" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="C108" s="32" t="n">
-        <v>34.9</v>
-      </c>
-      <c r="D108" s="32" t="n">
-        <v>36.05</v>
-      </c>
-      <c r="E108" s="32" t="n">
-        <v>36.467</v>
-      </c>
-      <c r="F108" s="32" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="G108" s="32" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="H108" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I108" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J108" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K108" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="L108" s="32" t="n">
-        <v>34.556</v>
-      </c>
-      <c r="M108" s="32" t="n">
-        <v>34.929</v>
-      </c>
-      <c r="N108" s="32" t="n">
-        <v>35.053</v>
-      </c>
-      <c r="O108" s="32" t="n">
-        <v>35.69</v>
-      </c>
-      <c r="P108" s="32" t="n">
-        <v>34.556</v>
-      </c>
-      <c r="Q108" s="34" t="inlineStr">
-        <is>
-          <t>Opp REB</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="31" t="inlineStr">
-        <is>
-          <t>AST</t>
-        </is>
-      </c>
-      <c r="B109" s="32" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="C109" s="32" t="n">
-        <v>21.533</v>
-      </c>
-      <c r="D109" s="32" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="E109" s="32" t="n">
-        <v>20.867</v>
-      </c>
-      <c r="F109" s="32" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="G109" s="32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="H109" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I109" s="32" t="inlineStr"/>
-      <c r="J109" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q109" s="34" t="inlineStr">
-        <is>
-          <t>Opp AST</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B110" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="C110" s="32" t="n">
-        <v>12.567</v>
-      </c>
-      <c r="D110" s="32" t="n">
-        <v>13.05</v>
-      </c>
-      <c r="E110" s="32" t="n">
-        <v>12.867</v>
-      </c>
-      <c r="F110" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="G110" s="32" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="H110" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I110" s="32" t="inlineStr"/>
-      <c r="J110" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q110" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="31" t="inlineStr">
-        <is>
-          <t>TOV</t>
-        </is>
-      </c>
-      <c r="B111" s="32" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="C111" s="32" t="n">
-        <v>12.733</v>
-      </c>
-      <c r="D111" s="32" t="n">
-        <v>13.35</v>
-      </c>
-      <c r="E111" s="32" t="n">
-        <v>13.733</v>
-      </c>
-      <c r="F111" s="32" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="G111" s="32" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H111" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
-        </is>
-      </c>
-      <c r="I111" s="32" t="inlineStr"/>
-      <c r="J111" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q111" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>

</xml_diff>

<commit_message>
data: hourly update 2026-07-13 18:46Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-13.xlsx
+++ b/data/output/workbook/2026-07-13.xlsx
@@ -363,7 +363,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12306300"/>
+    <ext cx="10125075" cy="12877800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 11:46</t>
+          <t>2026-07-13 14:46</t>
         </is>
       </c>
     </row>
@@ -1128,17 +1128,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Over 166.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.617</v>
+        <v>0.6268</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-161</v>
+        <v>-168</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1189,22 +1189,22 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.5389</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-125</v>
+        <v>-117</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Portland Fire @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -1260,14 +1260,14 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Connecticut Sun</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5438</v>
+        <v>0.5487</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-119</v>
+        <v>-122</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>100</v>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1306,37 +1306,37 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Phoenix Mercury @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Over 169.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5575</v>
+        <v>0.5187</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-126</v>
+        <v>-108</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1537,10 +1537,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4898</v>
+        <v>0.5006</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>104</v>
+        <v>-100</v>
       </c>
       <c r="H5" s="15" t="n"/>
       <c r="I5" s="13">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1601,10 +1601,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5102</v>
+        <v>0.4995</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="H6" s="15" t="n"/>
       <c r="I6" s="13">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 50.0% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1944,7 +1944,7 @@
         <v>106</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -2010,7 +2010,7 @@
         <v>-106</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2142,7 +2142,7 @@
         <v>-156</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>102</v>
+        <v>-105</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2330,17 +2330,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 170</t>
+          <t>Over 169.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5063</v>
+        <v>0.5187</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-103</v>
+        <v>-108</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-101</v>
+        <v>100</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -103). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2396,17 +2396,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 170</t>
+          <t>Under 169.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4703000000000001</v>
+        <v>0.4813</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 47.0% (fair +113). Your call.</t>
+          <t>Model 48.1% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2598,13 +2598,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4425</v>
+        <v>0.4513</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -2628,7 +2628,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 44.2% (fair +126). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -2664,13 +2664,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5575</v>
+        <v>0.5487</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-126</v>
+        <v>-122</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -2726,17 +2726,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Over 166.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.617</v>
+        <v>0.6268</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-161</v>
+        <v>-168</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2792,17 +2792,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 167.5</t>
+          <t>Under 166.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.383</v>
+        <v>0.3732</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 37.3% (fair +168). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -2868,7 +2868,7 @@
         <v>103</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-102</v>
+        <v>108</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -2994,13 +2994,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4562</v>
+        <v>0.4611</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -3060,13 +3060,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5438</v>
+        <v>0.5389</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-119</v>
+        <v>-117</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -3122,17 +3122,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Over 171.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.589124762254717</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-125</v>
+        <v>-143</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-104</v>
+        <v>111</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -3188,17 +3188,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 170.5</t>
+          <t>Under 171.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4441000000000001</v>
+        <v>0.410875237745283</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 41.1% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -3258,7 +3258,7 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5053400127859651</v>
+        <v>0.5051</v>
       </c>
       <c r="G27" s="14" t="n">
         <v>-102</v>
@@ -3324,13 +3324,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4946599872140349</v>
+        <v>0.4949</v>
       </c>
       <c r="G28" s="14" t="n">
         <v>102</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -5807,7 +5807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q107"/>
+  <dimension ref="A1:Q111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5824,765 +5824,493 @@
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="29" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
         <is>
           <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="30" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B78" s="30" t="inlineStr">
+      <c r="B82" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C78" s="30" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D78" s="30" t="inlineStr">
+      <c r="D82" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E78" s="30" t="inlineStr">
+      <c r="E82" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F78" s="30" t="inlineStr">
+      <c r="F82" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G78" s="30" t="inlineStr">
+      <c r="G82" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H78" s="30" t="inlineStr">
+      <c r="H82" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I78" s="30" t="inlineStr">
+      <c r="I82" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J78" s="30" t="inlineStr">
+      <c r="J82" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K78" s="30" t="inlineStr">
+      <c r="K82" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L78" s="30" t="inlineStr">
+      <c r="L82" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M78" s="30" t="inlineStr">
+      <c r="M82" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N78" s="30" t="inlineStr">
+      <c r="N82" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O78" s="30" t="inlineStr">
+      <c r="O82" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P78" s="30" t="inlineStr">
+      <c r="P82" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q78" s="30" t="inlineStr">
+      <c r="Q82" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="31" t="inlineStr">
-        <is>
-          <t>PPG</t>
-        </is>
-      </c>
-      <c r="B79" s="32" t="n">
-        <v>83</v>
-      </c>
-      <c r="C79" s="32" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="D79" s="32" t="n">
-        <v>83.05</v>
-      </c>
-      <c r="E79" s="32" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="F79" s="32" t="n">
-        <v>83</v>
-      </c>
-      <c r="G79" s="32" t="n">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="H79" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="n">
-        <v>72.75</v>
-      </c>
-      <c r="L79" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="M79" s="32" t="n">
-        <v>80</v>
-      </c>
-      <c r="N79" s="32" t="n">
-        <v>78.72199999999999</v>
-      </c>
-      <c r="O79" s="32" t="n">
-        <v>79</v>
-      </c>
-      <c r="P79" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="Q79" s="34" t="inlineStr">
-        <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B80" s="32" t="n">
-        <v>101.929</v>
-      </c>
-      <c r="C80" s="32" t="n">
-        <v>102.13</v>
-      </c>
-      <c r="D80" s="32" t="n">
-        <v>101.973</v>
-      </c>
-      <c r="E80" s="32" t="n">
-        <v>102.639</v>
-      </c>
-      <c r="F80" s="32" t="n">
-        <v>101.929</v>
-      </c>
-      <c r="G80" s="32" t="n">
-        <v>97.006</v>
-      </c>
-      <c r="H80" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I80" s="32" t="inlineStr"/>
-      <c r="J80" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K80" s="32" t="n">
-        <v>88.01600000000001</v>
-      </c>
-      <c r="L80" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="M80" s="32" t="n">
-        <v>97.129</v>
-      </c>
-      <c r="N80" s="32" t="n">
-        <v>96.706</v>
-      </c>
-      <c r="O80" s="32" t="n">
-        <v>98.628</v>
-      </c>
-      <c r="P80" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="Q80" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B81" s="32" t="n">
-        <v>0.476</v>
-      </c>
-      <c r="C81" s="32" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="D81" s="32" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="E81" s="32" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="F81" s="32" t="n">
-        <v>0.476</v>
-      </c>
-      <c r="G81" s="32" t="n">
-        <v>0.453</v>
-      </c>
-      <c r="H81" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K81" s="32" t="n">
-        <v>0.408</v>
-      </c>
-      <c r="L81" s="32" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="M81" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="N81" s="32" t="n">
-        <v>0.464</v>
-      </c>
-      <c r="O81" s="32" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="P81" s="32" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="Q81" s="34" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="31" t="inlineStr">
-        <is>
-          <t>2PT%</t>
-        </is>
-      </c>
-      <c r="B82" s="32" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="C82" s="32" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="D82" s="32" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="E82" s="32" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="F82" s="32" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="G82" s="32" t="n">
-        <v>0.454</v>
-      </c>
-      <c r="H82" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="L82" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="M82" s="32" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="N82" s="32" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="O82" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="P82" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="Q82" s="34" t="inlineStr">
-        <is>
-          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>0.32</v>
+        <v>83</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>0.33</v>
+        <v>82.3</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>0.315</v>
+        <v>83.05</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>0.318</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>0.32</v>
+        <v>83</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>0.293</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="H83" s="36" t="inlineStr">
         <is>
-          <t>12th</t>
+          <t>11th</t>
         </is>
       </c>
       <c r="I83" s="32" t="inlineStr"/>
       <c r="J83" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="K83" s="32" t="n">
-        <v>0.275</v>
+        <v>72.75</v>
       </c>
       <c r="L83" s="32" t="n">
-        <v>0.281</v>
+        <v>79.75</v>
       </c>
       <c r="M83" s="32" t="n">
-        <v>0.308</v>
+        <v>80</v>
       </c>
       <c r="N83" s="32" t="n">
-        <v>0.311</v>
+        <v>78.72199999999999</v>
       </c>
       <c r="O83" s="32" t="n">
-        <v>0.342</v>
+        <v>79</v>
       </c>
       <c r="P83" s="32" t="n">
-        <v>0.281</v>
+        <v>79.75</v>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>101.929</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>0.797</v>
+        <v>102.13</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>0.822</v>
+        <v>101.973</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>0.8070000000000001</v>
+        <v>102.639</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>101.929</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="H84" s="33" t="inlineStr">
-        <is>
-          <t>4th</t>
+        <v>97.006</v>
+      </c>
+      <c r="H84" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
-      <c r="J84" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J84" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K84" s="32" t="n">
+        <v>88.01600000000001</v>
+      </c>
+      <c r="L84" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="M84" s="32" t="n">
+        <v>97.129</v>
+      </c>
+      <c r="N84" s="32" t="n">
+        <v>96.706</v>
+      </c>
+      <c r="O84" s="32" t="n">
+        <v>98.628</v>
+      </c>
+      <c r="P84" s="32" t="n">
+        <v>95.66500000000001</v>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.476</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>80.69199999999999</v>
+        <v>0.491</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>81.45399999999999</v>
+        <v>0.486</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>81.39700000000001</v>
+        <v>0.488</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.476</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>79.672</v>
-      </c>
-      <c r="H85" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
+        <v>0.453</v>
+      </c>
+      <c r="H85" s="36" t="inlineStr">
+        <is>
+          <t>12th</t>
         </is>
       </c>
       <c r="I85" s="32" t="inlineStr"/>
-      <c r="J85" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J85" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K85" s="32" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="L85" s="32" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="M85" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="N85" s="32" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="O85" s="32" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="P85" s="32" t="n">
+        <v>0.441</v>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.543</v>
+        <v>0.467</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.54</v>
+        <v>0.48</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.54</v>
+        <v>0.486</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.547</v>
+        <v>0.488</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.543</v>
+        <v>0.467</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.519</v>
+        <v>0.454</v>
       </c>
       <c r="H86" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
-      <c r="J86" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J86" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K86" s="32" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="L86" s="32" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="M86" s="32" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="N86" s="32" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="O86" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="P86" s="32" t="n">
+        <v>0.449</v>
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>0.225</v>
+        <v>0.32</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>0.228</v>
+        <v>0.33</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>0.231</v>
+        <v>0.315</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>0.226</v>
+        <v>0.318</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>0.225</v>
+        <v>0.32</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>0.231</v>
+        <v>0.293</v>
       </c>
       <c r="H87" s="36" t="inlineStr">
         <is>
-          <t>10th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
-      <c r="J87" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J87" s="33" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K87" s="32" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="L87" s="32" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="M87" s="32" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="N87" s="32" t="n">
+        <v>0.311</v>
+      </c>
+      <c r="O87" s="32" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="P87" s="32" t="n">
+        <v>0.281</v>
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>31.2</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>34.167</v>
+        <v>0.797</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>34.5</v>
+        <v>0.822</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>32.867</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>31.2</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="H88" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>0.821</v>
+      </c>
+      <c r="H88" s="33" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
-      <c r="J88" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K88" s="32" t="n">
-        <v>30</v>
-      </c>
-      <c r="L88" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="M88" s="32" t="n">
-        <v>33.615</v>
-      </c>
-      <c r="N88" s="32" t="n">
-        <v>33.444</v>
-      </c>
-      <c r="O88" s="32" t="n">
-        <v>32.893</v>
-      </c>
-      <c r="P88" s="32" t="n">
-        <v>32.75</v>
+      <c r="J88" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>17.7</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>19.933</v>
+        <v>80.69199999999999</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>18.9</v>
+        <v>81.45399999999999</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>17.867</v>
+        <v>81.39700000000001</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>17.7</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="H89" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>79.672</v>
+      </c>
+      <c r="H89" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -6623,37 +6351,37 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>11.1</v>
+        <v>0.543</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>10.967</v>
+        <v>0.54</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>10.15</v>
+        <v>0.54</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>9.933</v>
+        <v>0.547</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>11.1</v>
+        <v>0.543</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="H90" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
+        <v>0.519</v>
+      </c>
+      <c r="H90" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
@@ -6694,37 +6422,37 @@
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B91" s="32" t="n">
-        <v>12.6</v>
+        <v>0.225</v>
       </c>
       <c r="C91" s="32" t="n">
-        <v>12.267</v>
+        <v>0.228</v>
       </c>
       <c r="D91" s="32" t="n">
-        <v>12.5</v>
+        <v>0.231</v>
       </c>
       <c r="E91" s="32" t="n">
-        <v>12.733</v>
+        <v>0.226</v>
       </c>
       <c r="F91" s="32" t="n">
-        <v>12.6</v>
+        <v>0.225</v>
       </c>
       <c r="G91" s="32" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="H91" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
+        <v>0.231</v>
+      </c>
+      <c r="H91" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
         </is>
       </c>
       <c r="I91" s="32" t="inlineStr"/>
@@ -6765,383 +6493,403 @@
       </c>
       <c r="Q91" s="34" t="inlineStr">
         <is>
-          <t>Opp TOV</t>
+          <t>Opp OREB%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="B92" s="32" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="C92" s="32" t="n">
+        <v>34.167</v>
+      </c>
+      <c r="D92" s="32" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="E92" s="32" t="n">
+        <v>32.867</v>
+      </c>
+      <c r="F92" s="32" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="G92" s="32" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="H92" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
+        </is>
+      </c>
+      <c r="I92" s="32" t="inlineStr"/>
+      <c r="J92" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K92" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="L92" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="M92" s="32" t="n">
+        <v>33.615</v>
+      </c>
+      <c r="N92" s="32" t="n">
+        <v>33.444</v>
+      </c>
+      <c r="O92" s="32" t="n">
+        <v>32.893</v>
+      </c>
+      <c r="P92" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="Q92" s="34" t="inlineStr">
+        <is>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="29" t="inlineStr">
-        <is>
-          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
+      <c r="A93" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="C93" s="32" t="n">
+        <v>19.933</v>
+      </c>
+      <c r="D93" s="32" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="E93" s="32" t="n">
+        <v>17.867</v>
+      </c>
+      <c r="F93" s="32" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G93" s="32" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="H93" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
+        </is>
+      </c>
+      <c r="I93" s="32" t="inlineStr"/>
+      <c r="J93" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q93" s="34" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B94" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C94" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D94" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E94" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F94" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G94" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H94" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I94" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J94" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K94" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L94" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M94" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N94" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O94" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P94" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q94" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A94" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B94" s="32" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C94" s="32" t="n">
+        <v>10.967</v>
+      </c>
+      <c r="D94" s="32" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="E94" s="32" t="n">
+        <v>9.933</v>
+      </c>
+      <c r="F94" s="32" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="G94" s="32" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H94" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="I94" s="32" t="inlineStr"/>
+      <c r="J94" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q94" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B95" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="C95" s="32" t="n">
-        <v>85.2</v>
+        <v>12.267</v>
       </c>
       <c r="D95" s="32" t="n">
-        <v>84.90000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="E95" s="32" t="n">
-        <v>85.867</v>
+        <v>12.733</v>
       </c>
       <c r="F95" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="G95" s="32" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="H95" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I95" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J95" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K95" s="32" t="n">
-        <v>89.8</v>
-      </c>
-      <c r="L95" s="32" t="n">
-        <v>86.77800000000001</v>
-      </c>
-      <c r="M95" s="32" t="n">
-        <v>87.786</v>
-      </c>
-      <c r="N95" s="32" t="n">
-        <v>84.36799999999999</v>
-      </c>
-      <c r="O95" s="32" t="n">
-        <v>82.655</v>
-      </c>
-      <c r="P95" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>13.4</v>
+      </c>
+      <c r="H95" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="inlineStr"/>
+      <c r="J95" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q95" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B96" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="C96" s="32" t="n">
-        <v>107.942</v>
-      </c>
-      <c r="D96" s="32" t="n">
-        <v>105.587</v>
-      </c>
-      <c r="E96" s="32" t="n">
-        <v>105.509</v>
-      </c>
-      <c r="F96" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="G96" s="32" t="n">
-        <v>115.565</v>
-      </c>
-      <c r="H96" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I96" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J96" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K96" s="32" t="n">
-        <v>113.552</v>
-      </c>
-      <c r="L96" s="32" t="n">
-        <v>108.265</v>
-      </c>
-      <c r="M96" s="32" t="n">
-        <v>109.197</v>
-      </c>
-      <c r="N96" s="32" t="n">
-        <v>104.078</v>
-      </c>
-      <c r="O96" s="32" t="n">
-        <v>102.45</v>
-      </c>
-      <c r="P96" s="32" t="n">
-        <v>108.265</v>
-      </c>
-      <c r="Q96" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp TOV</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B97" s="32" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="C97" s="32" t="n">
-        <v>0.544</v>
-      </c>
-      <c r="D97" s="32" t="n">
-        <v>0.533</v>
-      </c>
-      <c r="E97" s="32" t="n">
-        <v>0.535</v>
-      </c>
-      <c r="F97" s="32" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="G97" s="32" t="n">
-        <v>0.579</v>
-      </c>
-      <c r="H97" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I97" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J97" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K97" s="32" t="n">
-        <v>0.571</v>
-      </c>
-      <c r="L97" s="32" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="M97" s="32" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N97" s="32" t="n">
-        <v>0.506</v>
-      </c>
-      <c r="O97" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P97" s="32" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="Q97" s="34" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="31" t="inlineStr">
-        <is>
-          <t>2PT%</t>
-        </is>
-      </c>
-      <c r="B98" s="32" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="C98" s="32" t="n">
-        <v>0.534</v>
-      </c>
-      <c r="D98" s="32" t="n">
-        <v>0.543</v>
-      </c>
-      <c r="E98" s="32" t="n">
-        <v>0.549</v>
-      </c>
-      <c r="F98" s="32" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="G98" s="32" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="H98" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I98" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J98" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K98" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L98" s="32" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="M98" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N98" s="32" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="O98" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="P98" s="32" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="Q98" s="34" t="inlineStr">
-        <is>
-          <t>Opp 2PT%</t>
+      <c r="A98" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B98" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C98" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D98" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E98" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F98" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G98" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H98" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I98" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J98" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K98" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L98" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M98" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N98" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O98" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P98" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q98" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>0.373</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>0.374</v>
+        <v>85.2</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>0.343</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>0.347</v>
+        <v>85.867</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>0.373</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>0.382</v>
+        <v>94.2</v>
       </c>
       <c r="H99" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I99" s="32" t="inlineStr">
@@ -7155,403 +6903,379 @@
         </is>
       </c>
       <c r="K99" s="32" t="n">
-        <v>0.453</v>
+        <v>89.8</v>
       </c>
       <c r="L99" s="32" t="n">
-        <v>0.39</v>
+        <v>86.77800000000001</v>
       </c>
       <c r="M99" s="32" t="n">
-        <v>0.381</v>
+        <v>87.786</v>
       </c>
       <c r="N99" s="32" t="n">
-        <v>0.347</v>
+        <v>84.36799999999999</v>
       </c>
       <c r="O99" s="32" t="n">
-        <v>0.337</v>
+        <v>82.655</v>
       </c>
       <c r="P99" s="32" t="n">
-        <v>0.39</v>
+        <v>86.77800000000001</v>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>0.767</v>
+        <v>109.659</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>0.744</v>
+        <v>107.942</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>0.749</v>
+        <v>105.587</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>0.779</v>
+        <v>105.509</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>0.767</v>
+        <v>109.659</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>0.842</v>
+        <v>115.565</v>
       </c>
       <c r="H100" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="I100" s="32" t="inlineStr"/>
-      <c r="J100" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I100" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J100" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K100" s="32" t="n">
+        <v>113.552</v>
+      </c>
+      <c r="L100" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="M100" s="32" t="n">
+        <v>109.197</v>
+      </c>
+      <c r="N100" s="32" t="n">
+        <v>104.078</v>
+      </c>
+      <c r="O100" s="32" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="P100" s="32" t="n">
+        <v>108.265</v>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>81.724</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>79.247</v>
+        <v>0.544</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>80.62</v>
+        <v>0.533</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>81.736</v>
+        <v>0.535</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>81.724</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>82.304</v>
-      </c>
-      <c r="H101" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I101" s="32" t="inlineStr"/>
-      <c r="J101" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.579</v>
+      </c>
+      <c r="H101" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I101" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J101" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K101" s="32" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="L101" s="32" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="M101" s="32" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N101" s="32" t="n">
+        <v>0.506</v>
+      </c>
+      <c r="O101" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P101" s="32" t="n">
+        <v>0.545</v>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
-        <v>0.591</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="C102" s="32" t="n">
-        <v>0.57</v>
+        <v>0.534</v>
       </c>
       <c r="D102" s="32" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E102" s="32" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="F102" s="32" t="n">
         <v>0.5610000000000001</v>
       </c>
-      <c r="E102" s="32" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="F102" s="32" t="n">
-        <v>0.591</v>
-      </c>
       <c r="G102" s="32" t="n">
-        <v>0.613</v>
+        <v>0.582</v>
       </c>
       <c r="H102" s="33" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I102" s="32" t="inlineStr"/>
-      <c r="J102" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I102" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J102" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K102" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L102" s="32" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="M102" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N102" s="32" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="O102" s="32" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="P102" s="32" t="n">
+        <v>0.514</v>
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>0.265</v>
+        <v>0.373</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>0.255</v>
+        <v>0.374</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>0.253</v>
+        <v>0.343</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>0.245</v>
+        <v>0.347</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>0.265</v>
+        <v>0.373</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>0.287</v>
+        <v>0.382</v>
       </c>
       <c r="H103" s="33" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="I103" s="32" t="inlineStr"/>
-      <c r="J103" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I103" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J103" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K103" s="32" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="L103" s="32" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="M103" s="32" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="N103" s="32" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="O103" s="32" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="P103" s="32" t="n">
+        <v>0.39</v>
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>37.6</v>
+        <v>0.767</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>34.9</v>
+        <v>0.744</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>36.05</v>
+        <v>0.749</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>36.467</v>
+        <v>0.779</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>37.6</v>
+        <v>0.767</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>40.4</v>
+        <v>0.842</v>
       </c>
       <c r="H104" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I104" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J104" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K104" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="L104" s="32" t="n">
-        <v>34.556</v>
-      </c>
-      <c r="M104" s="32" t="n">
-        <v>34.929</v>
-      </c>
-      <c r="N104" s="32" t="n">
-        <v>35.053</v>
-      </c>
-      <c r="O104" s="32" t="n">
-        <v>35.69</v>
-      </c>
-      <c r="P104" s="32" t="n">
-        <v>34.556</v>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I104" s="32" t="inlineStr"/>
+      <c r="J104" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>21.1</v>
+        <v>81.724</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>21.533</v>
+        <v>79.247</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>21.1</v>
+        <v>80.62</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>20.867</v>
+        <v>81.736</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>21.1</v>
+        <v>81.724</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="H105" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
+        <v>82.304</v>
+      </c>
+      <c r="H105" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -7592,37 +7316,37 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>13</v>
+        <v>0.591</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>12.567</v>
+        <v>0.57</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>13.05</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>12.867</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>13</v>
+        <v>0.591</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>14.2</v>
+        <v>0.613</v>
       </c>
       <c r="H106" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I106" s="32" t="inlineStr"/>
@@ -7663,37 +7387,37 @@
       </c>
       <c r="Q106" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B107" s="32" t="n">
-        <v>14.8</v>
+        <v>0.265</v>
       </c>
       <c r="C107" s="32" t="n">
-        <v>12.733</v>
+        <v>0.255</v>
       </c>
       <c r="D107" s="32" t="n">
-        <v>13.35</v>
+        <v>0.253</v>
       </c>
       <c r="E107" s="32" t="n">
-        <v>13.733</v>
+        <v>0.245</v>
       </c>
       <c r="F107" s="32" t="n">
-        <v>14.8</v>
+        <v>0.265</v>
       </c>
       <c r="G107" s="32" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H107" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>0.287</v>
+      </c>
+      <c r="H107" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I107" s="32" t="inlineStr"/>
@@ -7733,6 +7457,282 @@
         </is>
       </c>
       <c r="Q107" s="34" t="inlineStr">
+        <is>
+          <t>Opp OREB%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="31" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="B108" s="32" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="C108" s="32" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="D108" s="32" t="n">
+        <v>36.05</v>
+      </c>
+      <c r="E108" s="32" t="n">
+        <v>36.467</v>
+      </c>
+      <c r="F108" s="32" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G108" s="32" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="H108" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I108" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J108" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K108" s="32" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="L108" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="M108" s="32" t="n">
+        <v>34.929</v>
+      </c>
+      <c r="N108" s="32" t="n">
+        <v>35.053</v>
+      </c>
+      <c r="O108" s="32" t="n">
+        <v>35.69</v>
+      </c>
+      <c r="P108" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="Q108" s="34" t="inlineStr">
+        <is>
+          <t>Opp REB</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="C109" s="32" t="n">
+        <v>21.533</v>
+      </c>
+      <c r="D109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="E109" s="32" t="n">
+        <v>20.867</v>
+      </c>
+      <c r="F109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="G109" s="32" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="H109" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I109" s="32" t="inlineStr"/>
+      <c r="J109" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q109" s="34" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C110" s="32" t="n">
+        <v>12.567</v>
+      </c>
+      <c r="D110" s="32" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="E110" s="32" t="n">
+        <v>12.867</v>
+      </c>
+      <c r="F110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="G110" s="32" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H110" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I110" s="32" t="inlineStr"/>
+      <c r="J110" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q110" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="31" t="inlineStr">
+        <is>
+          <t>TOV</t>
+        </is>
+      </c>
+      <c r="B111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C111" s="32" t="n">
+        <v>12.733</v>
+      </c>
+      <c r="D111" s="32" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="E111" s="32" t="n">
+        <v>13.733</v>
+      </c>
+      <c r="F111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="G111" s="32" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H111" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I111" s="32" t="inlineStr"/>
+      <c r="J111" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q111" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>

</xml_diff>

<commit_message>
data: hourly update 2026-07-13 19:30Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-13.xlsx
+++ b/data/output/workbook/2026-07-13.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 14:46</t>
+          <t>2026-07-13 15:29</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1179,12 +1179,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Portland Fire @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Connecticut Sun</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5389</v>
+        <v>0.5463</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-117</v>
+        <v>-120</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -1260,14 +1260,14 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5487</v>
+        <v>0.5414</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-122</v>
+        <v>-118</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>100</v>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 54.1% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1326,17 +1326,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 169.5</t>
+          <t>Over 170</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5187</v>
+        <v>0.4979</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-108</v>
+        <v>101</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 49.8% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1369,9 +1369,75 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Washington Mystics @ Toronto Tempo</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Washington Mystics +1.5</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>0.4923999999999999</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>103</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="I9" s="13">
+        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
+        <v/>
+      </c>
+      <c r="K9" s="17">
+        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L9" s="18">
+        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M9" s="12">
+        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.2% (fair +103). Your call.</t>
+        </is>
+      </c>
+      <c r="O9" s="15" t="n"/>
+      <c r="P9" s="16">
+        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J8">
+  <conditionalFormatting sqref="J5:J9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1812,7 +1878,7 @@
         <v>202</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -2010,7 +2076,7 @@
         <v>-106</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2076,7 +2142,7 @@
         <v>156</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2142,7 +2208,7 @@
         <v>-156</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-105</v>
+        <v>102</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2330,17 +2396,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 169.5</t>
+          <t>Over 170</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5187</v>
+        <v>0.4979</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-108</v>
+        <v>101</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2364,7 +2430,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 49.8% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2396,17 +2462,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 169.5</t>
+          <t>Under 170</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4813</v>
+        <v>0.4787</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>106</v>
+        <v>-102</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -2430,7 +2496,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2598,13 +2664,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4513</v>
+        <v>0.4537</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -2628,7 +2694,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.1% (fair +122). Your call.</t>
+          <t>Model 45.4% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -2664,10 +2730,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5487</v>
+        <v>0.5463</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-122</v>
+        <v>-120</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>100</v>
@@ -2694,7 +2760,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -2994,10 +3060,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4611</v>
+        <v>0.4586</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>-104</v>
@@ -3024,7 +3090,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 45.9% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -3060,13 +3126,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5389</v>
+        <v>0.5414</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-117</v>
+        <v>-118</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -3090,7 +3156,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 54.1% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -3258,10 +3324,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5051</v>
+        <v>0.5076000000000001</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-102</v>
+        <v>-103</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>100</v>
@@ -3288,7 +3354,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -3324,13 +3390,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4949</v>
+        <v>0.4923999999999999</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -3354,7 +3420,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-13 21:02Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-13.xlsx
+++ b/data/output/workbook/2026-07-13.xlsx
@@ -363,7 +363,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12877800"/>
+    <ext cx="10125075" cy="12649200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 15:29</t>
+          <t>2026-07-13 17:02</t>
         </is>
       </c>
     </row>
@@ -1128,14 +1128,14 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 166.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6268</v>
+        <v>0.6172</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-168</v>
+        <v>-161</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>-104</v>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 62.7% (fair -168). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1179,32 +1179,32 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5463</v>
+        <v>0.5632</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-120</v>
+        <v>-129</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.6% (fair -120). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1264,10 +1264,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5414</v>
+        <v>0.5426</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-118</v>
+        <v>-119</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>100</v>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1306,37 +1306,37 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Minnesota Lynx</t>
+          <t>Portland Fire @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 170</t>
+          <t>Connecticut Sun</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4979</v>
+        <v>0.5487</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>101</v>
+        <v>-122</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>107</v>
+        <v>-104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1372,37 +1372,37 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Phoenix Mercury @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics +1.5</t>
+          <t>Over 170</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4923999999999999</v>
+        <v>0.4985</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 49.9% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -1878,7 +1878,7 @@
         <v>202</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1944,7 +1944,7 @@
         <v>-202</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-115</v>
+        <v>-120</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -2000,17 +2000,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 182.5</t>
+          <t>Over 181.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4847500404119037</v>
+        <v>0.5082129373231845</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>106</v>
+        <v>-103</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -2066,17 +2066,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 182.5</t>
+          <t>Under 181.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5152499595880963</v>
+        <v>0.4917870626768155</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-106</v>
+        <v>103</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2142,7 +2142,7 @@
         <v>156</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2208,7 +2208,7 @@
         <v>-156</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2340,7 +2340,7 @@
         <v>-1157</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -2400,13 +2400,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4979</v>
+        <v>0.4985</v>
       </c>
       <c r="G13" s="14" t="n">
         <v>101</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 49.9% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2466,7 +2466,7 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4787</v>
+        <v>0.4781000000000001</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>109</v>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 47.9% (fair +109). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2664,10 +2664,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4537</v>
+        <v>0.4513</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>104</v>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.4% (fair +120). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -2730,13 +2730,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5463</v>
+        <v>0.5487</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-120</v>
+        <v>-122</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.6% (fair -120). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -2792,14 +2792,14 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 166.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.6268</v>
+        <v>0.6172</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-168</v>
+        <v>-161</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>-104</v>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 62.7% (fair -168). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2858,14 +2858,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 166.5</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3732</v>
+        <v>0.3828</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>104</v>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 37.3% (fair +168). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -3060,13 +3060,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4586</v>
+        <v>0.4574</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 45.7% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -3126,10 +3126,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5414</v>
+        <v>0.5426</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-118</v>
+        <v>-119</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>100</v>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -3188,17 +3188,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 171.5</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.589124762254717</v>
+        <v>0.5632</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-143</v>
+        <v>-129</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>111</v>
+        <v>-104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 58.9% (fair -143). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -3254,14 +3254,14 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 171.5</t>
+          <t>Under 170.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.410875237745283</v>
+        <v>0.4368</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>108</v>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 41.1% (fair +143). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5076000000000001</v>
+        <v>0.5051</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-103</v>
+        <v>-102</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>100</v>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -3390,13 +3390,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4923999999999999</v>
+        <v>0.4949</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -5873,7 +5873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q111"/>
+  <dimension ref="A1:Q109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5890,127 +5890,245 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="29" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B80" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C80" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D80" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E80" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F80" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G80" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H80" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I80" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J80" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K80" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L80" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M80" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N80" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O80" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P80" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q80" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
     <row r="81">
-      <c r="A81" s="29" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
+      <c r="A81" s="31" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>83</v>
+      </c>
+      <c r="C81" s="32" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="D81" s="32" t="n">
+        <v>83.05</v>
+      </c>
+      <c r="E81" s="32" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="F81" s="32" t="n">
+        <v>83</v>
+      </c>
+      <c r="G81" s="32" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="H81" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr"/>
+      <c r="J81" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="n">
+        <v>72.75</v>
+      </c>
+      <c r="L81" s="32" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="M81" s="32" t="n">
+        <v>80</v>
+      </c>
+      <c r="N81" s="32" t="n">
+        <v>78.72199999999999</v>
+      </c>
+      <c r="O81" s="32" t="n">
+        <v>79</v>
+      </c>
+      <c r="P81" s="32" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="Q81" s="34" t="inlineStr">
+        <is>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B82" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C82" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D82" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E82" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F82" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G82" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H82" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I82" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J82" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K82" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L82" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M82" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N82" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O82" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P82" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q82" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A82" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B82" s="32" t="n">
+        <v>101.929</v>
+      </c>
+      <c r="C82" s="32" t="n">
+        <v>102.13</v>
+      </c>
+      <c r="D82" s="32" t="n">
+        <v>101.973</v>
+      </c>
+      <c r="E82" s="32" t="n">
+        <v>102.639</v>
+      </c>
+      <c r="F82" s="32" t="n">
+        <v>101.929</v>
+      </c>
+      <c r="G82" s="32" t="n">
+        <v>97.006</v>
+      </c>
+      <c r="H82" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="inlineStr"/>
+      <c r="J82" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K82" s="32" t="n">
+        <v>88.01600000000001</v>
+      </c>
+      <c r="L82" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="M82" s="32" t="n">
+        <v>97.129</v>
+      </c>
+      <c r="N82" s="32" t="n">
+        <v>96.706</v>
+      </c>
+      <c r="O82" s="32" t="n">
+        <v>98.628</v>
+      </c>
+      <c r="P82" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="Q82" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>83</v>
+        <v>0.476</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>82.3</v>
+        <v>0.491</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>83.05</v>
+        <v>0.486</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>83.59999999999999</v>
+        <v>0.488</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>83</v>
+        <v>0.476</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>77.40000000000001</v>
+        <v>0.453</v>
       </c>
       <c r="H83" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I83" s="32" t="inlineStr"/>
@@ -6020,56 +6138,56 @@
         </is>
       </c>
       <c r="K83" s="32" t="n">
-        <v>72.75</v>
+        <v>0.408</v>
       </c>
       <c r="L83" s="32" t="n">
-        <v>79.75</v>
+        <v>0.441</v>
       </c>
       <c r="M83" s="32" t="n">
-        <v>80</v>
+        <v>0.461</v>
       </c>
       <c r="N83" s="32" t="n">
-        <v>78.72199999999999</v>
+        <v>0.464</v>
       </c>
       <c r="O83" s="32" t="n">
-        <v>79</v>
+        <v>0.481</v>
       </c>
       <c r="P83" s="32" t="n">
-        <v>79.75</v>
+        <v>0.441</v>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>101.929</v>
+        <v>0.467</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>102.13</v>
+        <v>0.48</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>101.973</v>
+        <v>0.486</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>102.639</v>
+        <v>0.488</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>101.929</v>
+        <v>0.467</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>97.006</v>
+        <v>0.454</v>
       </c>
       <c r="H84" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
@@ -6079,52 +6197,52 @@
         </is>
       </c>
       <c r="K84" s="32" t="n">
-        <v>88.01600000000001</v>
+        <v>0.404</v>
       </c>
       <c r="L84" s="32" t="n">
-        <v>95.66500000000001</v>
+        <v>0.449</v>
       </c>
       <c r="M84" s="32" t="n">
-        <v>97.129</v>
+        <v>0.456</v>
       </c>
       <c r="N84" s="32" t="n">
-        <v>96.706</v>
+        <v>0.463</v>
       </c>
       <c r="O84" s="32" t="n">
-        <v>98.628</v>
+        <v>0.461</v>
       </c>
       <c r="P84" s="32" t="n">
-        <v>95.66500000000001</v>
+        <v>0.449</v>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>0.476</v>
+        <v>0.32</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>0.491</v>
+        <v>0.33</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>0.486</v>
+        <v>0.315</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>0.488</v>
+        <v>0.318</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>0.476</v>
+        <v>0.32</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>0.453</v>
+        <v>0.293</v>
       </c>
       <c r="H85" s="36" t="inlineStr">
         <is>
@@ -6134,178 +6252,202 @@
       <c r="I85" s="32" t="inlineStr"/>
       <c r="J85" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="K85" s="32" t="n">
-        <v>0.408</v>
+        <v>0.275</v>
       </c>
       <c r="L85" s="32" t="n">
-        <v>0.441</v>
+        <v>0.281</v>
       </c>
       <c r="M85" s="32" t="n">
-        <v>0.461</v>
+        <v>0.308</v>
       </c>
       <c r="N85" s="32" t="n">
-        <v>0.464</v>
+        <v>0.311</v>
       </c>
       <c r="O85" s="32" t="n">
-        <v>0.481</v>
+        <v>0.342</v>
       </c>
       <c r="P85" s="32" t="n">
-        <v>0.441</v>
+        <v>0.281</v>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.467</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.48</v>
+        <v>0.797</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.486</v>
+        <v>0.822</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.488</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.467</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.454</v>
-      </c>
-      <c r="H86" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
+        <v>0.821</v>
+      </c>
+      <c r="H86" s="33" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
-      <c r="J86" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K86" s="32" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="L86" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="M86" s="32" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="N86" s="32" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="O86" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="P86" s="32" t="n">
-        <v>0.449</v>
+      <c r="J86" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>0.32</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>0.33</v>
+        <v>80.69199999999999</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>0.315</v>
+        <v>81.45399999999999</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>0.318</v>
+        <v>81.39700000000001</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>0.32</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="H87" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
+        <v>79.672</v>
+      </c>
+      <c r="H87" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
-      <c r="J87" s="33" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="K87" s="32" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="L87" s="32" t="n">
-        <v>0.281</v>
-      </c>
-      <c r="M87" s="32" t="n">
-        <v>0.308</v>
-      </c>
-      <c r="N87" s="32" t="n">
-        <v>0.311</v>
-      </c>
-      <c r="O87" s="32" t="n">
-        <v>0.342</v>
-      </c>
-      <c r="P87" s="32" t="n">
-        <v>0.281</v>
+      <c r="J87" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P87" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.543</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>0.797</v>
+        <v>0.54</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>0.822</v>
+        <v>0.54</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.547</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.543</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="H88" s="33" t="inlineStr">
-        <is>
-          <t>4th</t>
+        <v>0.519</v>
+      </c>
+      <c r="H88" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
@@ -6346,37 +6488,37 @@
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.225</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>80.69199999999999</v>
+        <v>0.228</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>81.45399999999999</v>
+        <v>0.231</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>81.39700000000001</v>
+        <v>0.226</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.225</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>79.672</v>
-      </c>
-      <c r="H89" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
+        <v>0.231</v>
+      </c>
+      <c r="H89" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -6417,108 +6559,96 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>0.543</v>
+        <v>31.2</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>0.54</v>
+        <v>34.167</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>0.54</v>
+        <v>34.5</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>0.547</v>
+        <v>32.867</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>0.543</v>
+        <v>31.2</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>0.519</v>
+        <v>29.6</v>
       </c>
       <c r="H90" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>13th</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
-      <c r="J90" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K90" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L90" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M90" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N90" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O90" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P90" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J90" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K90" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="L90" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="M90" s="32" t="n">
+        <v>33.615</v>
+      </c>
+      <c r="N90" s="32" t="n">
+        <v>33.444</v>
+      </c>
+      <c r="O90" s="32" t="n">
+        <v>32.893</v>
+      </c>
+      <c r="P90" s="32" t="n">
+        <v>32.75</v>
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B91" s="32" t="n">
-        <v>0.225</v>
+        <v>17.7</v>
       </c>
       <c r="C91" s="32" t="n">
-        <v>0.228</v>
+        <v>19.933</v>
       </c>
       <c r="D91" s="32" t="n">
-        <v>0.231</v>
+        <v>18.9</v>
       </c>
       <c r="E91" s="32" t="n">
-        <v>0.226</v>
+        <v>17.867</v>
       </c>
       <c r="F91" s="32" t="n">
-        <v>0.225</v>
+        <v>17.7</v>
       </c>
       <c r="G91" s="32" t="n">
-        <v>0.231</v>
+        <v>16.4</v>
       </c>
       <c r="H91" s="36" t="inlineStr">
         <is>
-          <t>10th</t>
+          <t>13th</t>
         </is>
       </c>
       <c r="I91" s="32" t="inlineStr"/>
@@ -6559,96 +6689,108 @@
       </c>
       <c r="Q91" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B92" s="32" t="n">
-        <v>31.2</v>
+        <v>11.1</v>
       </c>
       <c r="C92" s="32" t="n">
-        <v>34.167</v>
+        <v>10.967</v>
       </c>
       <c r="D92" s="32" t="n">
-        <v>34.5</v>
+        <v>10.15</v>
       </c>
       <c r="E92" s="32" t="n">
-        <v>32.867</v>
+        <v>9.933</v>
       </c>
       <c r="F92" s="32" t="n">
-        <v>31.2</v>
+        <v>11.1</v>
       </c>
       <c r="G92" s="32" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="H92" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>11.4</v>
+      </c>
+      <c r="H92" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
         </is>
       </c>
       <c r="I92" s="32" t="inlineStr"/>
-      <c r="J92" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K92" s="32" t="n">
-        <v>30</v>
-      </c>
-      <c r="L92" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="M92" s="32" t="n">
-        <v>33.615</v>
-      </c>
-      <c r="N92" s="32" t="n">
-        <v>33.444</v>
-      </c>
-      <c r="O92" s="32" t="n">
-        <v>32.893</v>
-      </c>
-      <c r="P92" s="32" t="n">
-        <v>32.75</v>
+      <c r="J92" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K92" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L92" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M92" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N92" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O92" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P92" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q92" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B93" s="32" t="n">
-        <v>17.7</v>
+        <v>12.6</v>
       </c>
       <c r="C93" s="32" t="n">
-        <v>19.933</v>
+        <v>12.267</v>
       </c>
       <c r="D93" s="32" t="n">
-        <v>18.9</v>
+        <v>12.5</v>
       </c>
       <c r="E93" s="32" t="n">
-        <v>17.867</v>
+        <v>12.733</v>
       </c>
       <c r="F93" s="32" t="n">
-        <v>17.7</v>
+        <v>12.6</v>
       </c>
       <c r="G93" s="32" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="H93" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>13.4</v>
+      </c>
+      <c r="H93" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I93" s="32" t="inlineStr"/>
@@ -6689,269 +6831,253 @@
       </c>
       <c r="Q93" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B94" s="32" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="C94" s="32" t="n">
-        <v>10.967</v>
-      </c>
-      <c r="D94" s="32" t="n">
-        <v>10.15</v>
-      </c>
-      <c r="E94" s="32" t="n">
-        <v>9.933</v>
-      </c>
-      <c r="F94" s="32" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="G94" s="32" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="H94" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="I94" s="32" t="inlineStr"/>
-      <c r="J94" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q94" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TOV</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="31" t="inlineStr">
-        <is>
-          <t>TOV</t>
-        </is>
-      </c>
-      <c r="B95" s="32" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="C95" s="32" t="n">
-        <v>12.267</v>
-      </c>
-      <c r="D95" s="32" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="E95" s="32" t="n">
-        <v>12.733</v>
-      </c>
-      <c r="F95" s="32" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="G95" s="32" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="H95" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I95" s="32" t="inlineStr"/>
-      <c r="J95" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P95" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q95" s="34" t="inlineStr">
-        <is>
-          <t>Opp TOV</t>
+      <c r="A95" s="29" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B96" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C96" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D96" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E96" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F96" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G96" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H96" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I96" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J96" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K96" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L96" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M96" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N96" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O96" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P96" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q96" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="29" t="inlineStr">
-        <is>
-          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
+      <c r="A97" s="31" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="B97" s="32" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="C97" s="32" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="D97" s="32" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="E97" s="32" t="n">
+        <v>85.867</v>
+      </c>
+      <c r="F97" s="32" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="G97" s="32" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="H97" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I97" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J97" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K97" s="32" t="n">
+        <v>89.8</v>
+      </c>
+      <c r="L97" s="32" t="n">
+        <v>86.77800000000001</v>
+      </c>
+      <c r="M97" s="32" t="n">
+        <v>87.786</v>
+      </c>
+      <c r="N97" s="32" t="n">
+        <v>84.36799999999999</v>
+      </c>
+      <c r="O97" s="32" t="n">
+        <v>82.655</v>
+      </c>
+      <c r="P97" s="32" t="n">
+        <v>86.77800000000001</v>
+      </c>
+      <c r="Q97" s="34" t="inlineStr">
+        <is>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B98" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C98" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D98" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E98" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F98" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G98" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H98" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I98" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J98" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K98" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L98" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M98" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N98" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O98" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P98" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q98" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A98" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B98" s="32" t="n">
+        <v>109.659</v>
+      </c>
+      <c r="C98" s="32" t="n">
+        <v>107.942</v>
+      </c>
+      <c r="D98" s="32" t="n">
+        <v>105.587</v>
+      </c>
+      <c r="E98" s="32" t="n">
+        <v>105.509</v>
+      </c>
+      <c r="F98" s="32" t="n">
+        <v>109.659</v>
+      </c>
+      <c r="G98" s="32" t="n">
+        <v>115.565</v>
+      </c>
+      <c r="H98" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I98" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J98" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K98" s="32" t="n">
+        <v>113.552</v>
+      </c>
+      <c r="L98" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="M98" s="32" t="n">
+        <v>109.197</v>
+      </c>
+      <c r="N98" s="32" t="n">
+        <v>104.078</v>
+      </c>
+      <c r="O98" s="32" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="P98" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="Q98" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>85.2</v>
+        <v>0.544</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>84.90000000000001</v>
+        <v>0.533</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>85.867</v>
+        <v>0.535</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>94.2</v>
+        <v>0.579</v>
       </c>
       <c r="H99" s="33" t="inlineStr">
         <is>
@@ -6969,52 +7095,52 @@
         </is>
       </c>
       <c r="K99" s="32" t="n">
-        <v>89.8</v>
+        <v>0.571</v>
       </c>
       <c r="L99" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>0.545</v>
       </c>
       <c r="M99" s="32" t="n">
-        <v>87.786</v>
+        <v>0.53</v>
       </c>
       <c r="N99" s="32" t="n">
-        <v>84.36799999999999</v>
+        <v>0.506</v>
       </c>
       <c r="O99" s="32" t="n">
-        <v>82.655</v>
+        <v>0.5</v>
       </c>
       <c r="P99" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>0.545</v>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>109.659</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>107.942</v>
+        <v>0.534</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>105.587</v>
+        <v>0.543</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>105.509</v>
+        <v>0.549</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>109.659</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>115.565</v>
+        <v>0.582</v>
       </c>
       <c r="H100" s="33" t="inlineStr">
         <is>
@@ -7023,65 +7149,65 @@
       </c>
       <c r="I100" s="32" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="J100" s="36" t="inlineStr">
         <is>
-          <t>14th</t>
+          <t>10th</t>
         </is>
       </c>
       <c r="K100" s="32" t="n">
-        <v>113.552</v>
+        <v>0.5</v>
       </c>
       <c r="L100" s="32" t="n">
-        <v>108.265</v>
+        <v>0.514</v>
       </c>
       <c r="M100" s="32" t="n">
-        <v>109.197</v>
+        <v>0.5</v>
       </c>
       <c r="N100" s="32" t="n">
-        <v>104.078</v>
+        <v>0.494</v>
       </c>
       <c r="O100" s="32" t="n">
-        <v>102.45</v>
+        <v>0.497</v>
       </c>
       <c r="P100" s="32" t="n">
-        <v>108.265</v>
+        <v>0.514</v>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.373</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>0.544</v>
+        <v>0.374</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>0.533</v>
+        <v>0.343</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>0.535</v>
+        <v>0.347</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.373</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>0.579</v>
+        <v>0.382</v>
       </c>
       <c r="H101" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I101" s="32" t="inlineStr">
@@ -7095,182 +7221,198 @@
         </is>
       </c>
       <c r="K101" s="32" t="n">
-        <v>0.571</v>
+        <v>0.453</v>
       </c>
       <c r="L101" s="32" t="n">
-        <v>0.545</v>
+        <v>0.39</v>
       </c>
       <c r="M101" s="32" t="n">
-        <v>0.53</v>
+        <v>0.381</v>
       </c>
       <c r="N101" s="32" t="n">
-        <v>0.506</v>
+        <v>0.347</v>
       </c>
       <c r="O101" s="32" t="n">
-        <v>0.5</v>
+        <v>0.337</v>
       </c>
       <c r="P101" s="32" t="n">
-        <v>0.545</v>
+        <v>0.39</v>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.767</v>
       </c>
       <c r="C102" s="32" t="n">
-        <v>0.534</v>
+        <v>0.744</v>
       </c>
       <c r="D102" s="32" t="n">
-        <v>0.543</v>
+        <v>0.749</v>
       </c>
       <c r="E102" s="32" t="n">
-        <v>0.549</v>
+        <v>0.779</v>
       </c>
       <c r="F102" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.767</v>
       </c>
       <c r="G102" s="32" t="n">
-        <v>0.582</v>
+        <v>0.842</v>
       </c>
       <c r="H102" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I102" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J102" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K102" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L102" s="32" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="M102" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N102" s="32" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="O102" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="P102" s="32" t="n">
-        <v>0.514</v>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I102" s="32" t="inlineStr"/>
+      <c r="J102" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>0.373</v>
+        <v>81.724</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>0.374</v>
+        <v>79.247</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>0.343</v>
+        <v>80.62</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>0.347</v>
+        <v>81.736</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>0.373</v>
+        <v>81.724</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>0.382</v>
-      </c>
-      <c r="H103" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I103" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J103" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K103" s="32" t="n">
-        <v>0.453</v>
-      </c>
-      <c r="L103" s="32" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="M103" s="32" t="n">
-        <v>0.381</v>
-      </c>
-      <c r="N103" s="32" t="n">
-        <v>0.347</v>
-      </c>
-      <c r="O103" s="32" t="n">
-        <v>0.337</v>
-      </c>
-      <c r="P103" s="32" t="n">
-        <v>0.39</v>
+        <v>82.304</v>
+      </c>
+      <c r="H103" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I103" s="32" t="inlineStr"/>
+      <c r="J103" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P103" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>0.767</v>
+        <v>0.591</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>0.744</v>
+        <v>0.57</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>0.749</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>0.779</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>0.767</v>
+        <v>0.591</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>0.842</v>
+        <v>0.613</v>
       </c>
       <c r="H104" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I104" s="32" t="inlineStr"/>
@@ -7311,37 +7453,37 @@
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>81.724</v>
+        <v>0.265</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>79.247</v>
+        <v>0.255</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>80.62</v>
+        <v>0.253</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>81.736</v>
+        <v>0.245</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>81.724</v>
+        <v>0.265</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>82.304</v>
-      </c>
-      <c r="H105" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
+        <v>0.287</v>
+      </c>
+      <c r="H105" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -7382,108 +7524,100 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>0.591</v>
+        <v>37.6</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>0.57</v>
+        <v>34.9</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>36.05</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>0.5649999999999999</v>
+        <v>36.467</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>0.591</v>
+        <v>37.6</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>0.613</v>
+        <v>40.4</v>
       </c>
       <c r="H106" s="33" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I106" s="32" t="inlineStr"/>
-      <c r="J106" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K106" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L106" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M106" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N106" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O106" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P106" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I106" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J106" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K106" s="32" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="L106" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="M106" s="32" t="n">
+        <v>34.929</v>
+      </c>
+      <c r="N106" s="32" t="n">
+        <v>35.053</v>
+      </c>
+      <c r="O106" s="32" t="n">
+        <v>35.69</v>
+      </c>
+      <c r="P106" s="32" t="n">
+        <v>34.556</v>
       </c>
       <c r="Q106" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B107" s="32" t="n">
-        <v>0.265</v>
+        <v>21.1</v>
       </c>
       <c r="C107" s="32" t="n">
-        <v>0.255</v>
+        <v>21.533</v>
       </c>
       <c r="D107" s="32" t="n">
-        <v>0.253</v>
+        <v>21.1</v>
       </c>
       <c r="E107" s="32" t="n">
-        <v>0.245</v>
+        <v>20.867</v>
       </c>
       <c r="F107" s="32" t="n">
-        <v>0.265</v>
+        <v>21.1</v>
       </c>
       <c r="G107" s="32" t="n">
-        <v>0.287</v>
+        <v>23.2</v>
       </c>
       <c r="H107" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I107" s="32" t="inlineStr"/>
@@ -7524,100 +7658,108 @@
       </c>
       <c r="Q107" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B108" s="32" t="n">
-        <v>37.6</v>
+        <v>13</v>
       </c>
       <c r="C108" s="32" t="n">
-        <v>34.9</v>
+        <v>12.567</v>
       </c>
       <c r="D108" s="32" t="n">
-        <v>36.05</v>
+        <v>13.05</v>
       </c>
       <c r="E108" s="32" t="n">
-        <v>36.467</v>
+        <v>12.867</v>
       </c>
       <c r="F108" s="32" t="n">
-        <v>37.6</v>
+        <v>13</v>
       </c>
       <c r="G108" s="32" t="n">
-        <v>40.4</v>
+        <v>14.2</v>
       </c>
       <c r="H108" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I108" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J108" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K108" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="L108" s="32" t="n">
-        <v>34.556</v>
-      </c>
-      <c r="M108" s="32" t="n">
-        <v>34.929</v>
-      </c>
-      <c r="N108" s="32" t="n">
-        <v>35.053</v>
-      </c>
-      <c r="O108" s="32" t="n">
-        <v>35.69</v>
-      </c>
-      <c r="P108" s="32" t="n">
-        <v>34.556</v>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I108" s="32" t="inlineStr"/>
+      <c r="J108" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K108" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L108" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M108" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N108" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O108" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P108" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q108" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B109" s="32" t="n">
-        <v>21.1</v>
+        <v>14.8</v>
       </c>
       <c r="C109" s="32" t="n">
-        <v>21.533</v>
+        <v>12.733</v>
       </c>
       <c r="D109" s="32" t="n">
-        <v>21.1</v>
+        <v>13.35</v>
       </c>
       <c r="E109" s="32" t="n">
-        <v>20.867</v>
+        <v>13.733</v>
       </c>
       <c r="F109" s="32" t="n">
-        <v>21.1</v>
+        <v>14.8</v>
       </c>
       <c r="G109" s="32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="H109" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
+        <v>14.4</v>
+      </c>
+      <c r="H109" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
         </is>
       </c>
       <c r="I109" s="32" t="inlineStr"/>
@@ -7657,148 +7799,6 @@
         </is>
       </c>
       <c r="Q109" s="34" t="inlineStr">
-        <is>
-          <t>Opp AST</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B110" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="C110" s="32" t="n">
-        <v>12.567</v>
-      </c>
-      <c r="D110" s="32" t="n">
-        <v>13.05</v>
-      </c>
-      <c r="E110" s="32" t="n">
-        <v>12.867</v>
-      </c>
-      <c r="F110" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="G110" s="32" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="H110" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I110" s="32" t="inlineStr"/>
-      <c r="J110" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q110" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="31" t="inlineStr">
-        <is>
-          <t>TOV</t>
-        </is>
-      </c>
-      <c r="B111" s="32" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="C111" s="32" t="n">
-        <v>12.733</v>
-      </c>
-      <c r="D111" s="32" t="n">
-        <v>13.35</v>
-      </c>
-      <c r="E111" s="32" t="n">
-        <v>13.733</v>
-      </c>
-      <c r="F111" s="32" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="G111" s="32" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H111" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
-        </is>
-      </c>
-      <c r="I111" s="32" t="inlineStr"/>
-      <c r="J111" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P111" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q111" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>

</xml_diff>

<commit_message>
data: hourly update 2026-07-13 23:03Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-13.xlsx
+++ b/data/output/workbook/2026-07-13.xlsx
@@ -363,7 +363,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12649200"/>
+    <ext cx="10125075" cy="12306300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 17:02</t>
+          <t>2026-07-13 19:02</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -1128,14 +1128,14 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Over 170.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6172</v>
+        <v>0.5632</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-161</v>
+        <v>-129</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>-104</v>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1189,22 +1189,22 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5632</v>
+        <v>0.5389</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-129</v>
+        <v>-117</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Toronto Tempo</t>
+          <t>Portland Fire @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -1260,14 +1260,14 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Connecticut Sun</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5426</v>
+        <v>0.5463</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-119</v>
+        <v>-120</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>100</v>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1306,37 +1306,37 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Connecticut Sun</t>
+          <t>Phoenix Mercury @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Over 169.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5487</v>
+        <v>0.5162</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-122</v>
+        <v>-107</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1369,75 +1369,9 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury @ Minnesota Lynx</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>01:00</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Over 170</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>0.4985</v>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>101</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>106</v>
-      </c>
-      <c r="I9" s="13">
-        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
-        <v/>
-      </c>
-      <c r="J9" s="16">
-        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
-        <v/>
-      </c>
-      <c r="K9" s="17">
-        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L9" s="18">
-        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M9" s="12">
-        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N9" s="19" t="inlineStr">
-        <is>
-          <t>Model 49.9% (fair +101). Your call.</t>
-        </is>
-      </c>
-      <c r="O9" s="15" t="n"/>
-      <c r="P9" s="16">
-        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J9">
+  <conditionalFormatting sqref="J5:J8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1878,7 +1812,7 @@
         <v>202</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>317</v>
+        <v>330</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -2000,17 +1934,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 181.5</t>
+          <t>Over 182.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5082129373231845</v>
+        <v>0.4847500404119037</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-103</v>
+        <v>106</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -2034,7 +1968,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -2066,17 +2000,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 181.5</t>
+          <t>Under 182.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4917870626768155</v>
+        <v>0.5152499595880963</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>103</v>
+        <v>-106</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2100,7 +2034,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2142,7 +2076,7 @@
         <v>156</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2208,7 +2142,7 @@
         <v>-156</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2396,17 +2330,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 170</t>
+          <t>Over 169.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4985</v>
+        <v>0.5162</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>101</v>
+        <v>-107</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2430,7 +2364,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +101). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2462,17 +2396,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 170</t>
+          <t>Under 169.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4781000000000001</v>
+        <v>0.4838</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -2496,7 +2430,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2538,7 +2472,7 @@
         <v>102</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -2604,7 +2538,7 @@
         <v>-102</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -2664,10 +2598,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4513</v>
+        <v>0.4537</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>104</v>
@@ -2694,7 +2628,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.1% (fair +122). Your call.</t>
+          <t>Model 45.4% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -2730,13 +2664,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5487</v>
+        <v>0.5463</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-122</v>
+        <v>-120</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -2760,7 +2694,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -2792,17 +2726,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Over 168.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.6172</v>
+        <v>0.7045896324040164</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-161</v>
+        <v>-239</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-104</v>
+        <v>110</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -2826,7 +2760,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 70.5% (fair -239). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2858,14 +2792,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 167.5</t>
+          <t>Under 168.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3828</v>
+        <v>0.2954103675959836</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>161</v>
+        <v>239</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>104</v>
@@ -2892,7 +2826,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 29.5% (fair +239). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -2934,7 +2868,7 @@
         <v>103</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -3000,7 +2934,7 @@
         <v>-103</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -3060,13 +2994,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4574</v>
+        <v>0.4611</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-102</v>
+        <v>-104</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -3090,7 +3024,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -3126,13 +3060,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5426</v>
+        <v>0.5389</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-119</v>
+        <v>-117</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -3156,7 +3090,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -5873,7 +5807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q109"/>
+  <dimension ref="A1:Q107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5890,127 +5824,245 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B78" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C78" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D78" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E78" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F78" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G78" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H78" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I78" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J78" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K78" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L78" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M78" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N78" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O78" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P78" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q78" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
     <row r="79">
-      <c r="A79" s="29" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
+      <c r="A79" s="31" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="B79" s="32" t="n">
+        <v>83</v>
+      </c>
+      <c r="C79" s="32" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="D79" s="32" t="n">
+        <v>83.05</v>
+      </c>
+      <c r="E79" s="32" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="F79" s="32" t="n">
+        <v>83</v>
+      </c>
+      <c r="G79" s="32" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="H79" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I79" s="32" t="inlineStr"/>
+      <c r="J79" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="n">
+        <v>72.75</v>
+      </c>
+      <c r="L79" s="32" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="M79" s="32" t="n">
+        <v>80</v>
+      </c>
+      <c r="N79" s="32" t="n">
+        <v>78.72199999999999</v>
+      </c>
+      <c r="O79" s="32" t="n">
+        <v>79</v>
+      </c>
+      <c r="P79" s="32" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="Q79" s="34" t="inlineStr">
+        <is>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B80" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C80" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D80" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E80" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F80" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G80" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H80" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I80" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J80" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K80" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L80" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M80" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N80" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O80" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P80" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q80" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A80" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B80" s="32" t="n">
+        <v>101.929</v>
+      </c>
+      <c r="C80" s="32" t="n">
+        <v>102.13</v>
+      </c>
+      <c r="D80" s="32" t="n">
+        <v>101.973</v>
+      </c>
+      <c r="E80" s="32" t="n">
+        <v>102.639</v>
+      </c>
+      <c r="F80" s="32" t="n">
+        <v>101.929</v>
+      </c>
+      <c r="G80" s="32" t="n">
+        <v>97.006</v>
+      </c>
+      <c r="H80" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr"/>
+      <c r="J80" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K80" s="32" t="n">
+        <v>88.01600000000001</v>
+      </c>
+      <c r="L80" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="M80" s="32" t="n">
+        <v>97.129</v>
+      </c>
+      <c r="N80" s="32" t="n">
+        <v>96.706</v>
+      </c>
+      <c r="O80" s="32" t="n">
+        <v>98.628</v>
+      </c>
+      <c r="P80" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="Q80" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B81" s="32" t="n">
-        <v>83</v>
+        <v>0.476</v>
       </c>
       <c r="C81" s="32" t="n">
-        <v>82.3</v>
+        <v>0.491</v>
       </c>
       <c r="D81" s="32" t="n">
-        <v>83.05</v>
+        <v>0.486</v>
       </c>
       <c r="E81" s="32" t="n">
-        <v>83.59999999999999</v>
+        <v>0.488</v>
       </c>
       <c r="F81" s="32" t="n">
-        <v>83</v>
+        <v>0.476</v>
       </c>
       <c r="G81" s="32" t="n">
-        <v>77.40000000000001</v>
+        <v>0.453</v>
       </c>
       <c r="H81" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I81" s="32" t="inlineStr"/>
@@ -6020,56 +6072,56 @@
         </is>
       </c>
       <c r="K81" s="32" t="n">
-        <v>72.75</v>
+        <v>0.408</v>
       </c>
       <c r="L81" s="32" t="n">
-        <v>79.75</v>
+        <v>0.441</v>
       </c>
       <c r="M81" s="32" t="n">
-        <v>80</v>
+        <v>0.461</v>
       </c>
       <c r="N81" s="32" t="n">
-        <v>78.72199999999999</v>
+        <v>0.464</v>
       </c>
       <c r="O81" s="32" t="n">
-        <v>79</v>
+        <v>0.481</v>
       </c>
       <c r="P81" s="32" t="n">
-        <v>79.75</v>
+        <v>0.441</v>
       </c>
       <c r="Q81" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B82" s="32" t="n">
-        <v>101.929</v>
+        <v>0.467</v>
       </c>
       <c r="C82" s="32" t="n">
-        <v>102.13</v>
+        <v>0.48</v>
       </c>
       <c r="D82" s="32" t="n">
-        <v>101.973</v>
+        <v>0.486</v>
       </c>
       <c r="E82" s="32" t="n">
-        <v>102.639</v>
+        <v>0.488</v>
       </c>
       <c r="F82" s="32" t="n">
-        <v>101.929</v>
+        <v>0.467</v>
       </c>
       <c r="G82" s="32" t="n">
-        <v>97.006</v>
+        <v>0.454</v>
       </c>
       <c r="H82" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I82" s="32" t="inlineStr"/>
@@ -6079,52 +6131,52 @@
         </is>
       </c>
       <c r="K82" s="32" t="n">
-        <v>88.01600000000001</v>
+        <v>0.404</v>
       </c>
       <c r="L82" s="32" t="n">
-        <v>95.66500000000001</v>
+        <v>0.449</v>
       </c>
       <c r="M82" s="32" t="n">
-        <v>97.129</v>
+        <v>0.456</v>
       </c>
       <c r="N82" s="32" t="n">
-        <v>96.706</v>
+        <v>0.463</v>
       </c>
       <c r="O82" s="32" t="n">
-        <v>98.628</v>
+        <v>0.461</v>
       </c>
       <c r="P82" s="32" t="n">
-        <v>95.66500000000001</v>
+        <v>0.449</v>
       </c>
       <c r="Q82" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>0.476</v>
+        <v>0.32</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>0.491</v>
+        <v>0.33</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>0.486</v>
+        <v>0.315</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>0.488</v>
+        <v>0.318</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>0.476</v>
+        <v>0.32</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>0.453</v>
+        <v>0.293</v>
       </c>
       <c r="H83" s="36" t="inlineStr">
         <is>
@@ -6134,178 +6186,202 @@
       <c r="I83" s="32" t="inlineStr"/>
       <c r="J83" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="K83" s="32" t="n">
-        <v>0.408</v>
+        <v>0.275</v>
       </c>
       <c r="L83" s="32" t="n">
-        <v>0.441</v>
+        <v>0.281</v>
       </c>
       <c r="M83" s="32" t="n">
-        <v>0.461</v>
+        <v>0.308</v>
       </c>
       <c r="N83" s="32" t="n">
-        <v>0.464</v>
+        <v>0.311</v>
       </c>
       <c r="O83" s="32" t="n">
-        <v>0.481</v>
+        <v>0.342</v>
       </c>
       <c r="P83" s="32" t="n">
-        <v>0.441</v>
+        <v>0.281</v>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>0.467</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>0.48</v>
+        <v>0.797</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>0.486</v>
+        <v>0.822</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>0.488</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>0.467</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>0.454</v>
-      </c>
-      <c r="H84" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
+        <v>0.821</v>
+      </c>
+      <c r="H84" s="33" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
-      <c r="J84" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K84" s="32" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="L84" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="M84" s="32" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="N84" s="32" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="O84" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="P84" s="32" t="n">
-        <v>0.449</v>
+      <c r="J84" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>0.32</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>0.33</v>
+        <v>80.69199999999999</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>0.315</v>
+        <v>81.45399999999999</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>0.318</v>
+        <v>81.39700000000001</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>0.32</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="H85" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
+        <v>79.672</v>
+      </c>
+      <c r="H85" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
         </is>
       </c>
       <c r="I85" s="32" t="inlineStr"/>
-      <c r="J85" s="33" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="K85" s="32" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="L85" s="32" t="n">
-        <v>0.281</v>
-      </c>
-      <c r="M85" s="32" t="n">
-        <v>0.308</v>
-      </c>
-      <c r="N85" s="32" t="n">
-        <v>0.311</v>
-      </c>
-      <c r="O85" s="32" t="n">
-        <v>0.342</v>
-      </c>
-      <c r="P85" s="32" t="n">
-        <v>0.281</v>
+      <c r="J85" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.543</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.797</v>
+        <v>0.54</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.822</v>
+        <v>0.54</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.547</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.543</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="H86" s="33" t="inlineStr">
-        <is>
-          <t>4th</t>
+        <v>0.519</v>
+      </c>
+      <c r="H86" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
@@ -6346,37 +6422,37 @@
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.225</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>80.69199999999999</v>
+        <v>0.228</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>81.45399999999999</v>
+        <v>0.231</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>81.39700000000001</v>
+        <v>0.226</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.225</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>79.672</v>
-      </c>
-      <c r="H87" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
+        <v>0.231</v>
+      </c>
+      <c r="H87" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
@@ -6417,108 +6493,96 @@
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>0.543</v>
+        <v>31.2</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>0.54</v>
+        <v>34.167</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>0.54</v>
+        <v>34.5</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>0.547</v>
+        <v>32.867</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>0.543</v>
+        <v>31.2</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>0.519</v>
+        <v>29.6</v>
       </c>
       <c r="H88" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>13th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
-      <c r="J88" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P88" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J88" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K88" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="L88" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="M88" s="32" t="n">
+        <v>33.615</v>
+      </c>
+      <c r="N88" s="32" t="n">
+        <v>33.444</v>
+      </c>
+      <c r="O88" s="32" t="n">
+        <v>32.893</v>
+      </c>
+      <c r="P88" s="32" t="n">
+        <v>32.75</v>
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>0.225</v>
+        <v>17.7</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>0.228</v>
+        <v>19.933</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>0.231</v>
+        <v>18.9</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>0.226</v>
+        <v>17.867</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>0.225</v>
+        <v>17.7</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>0.231</v>
+        <v>16.4</v>
       </c>
       <c r="H89" s="36" t="inlineStr">
         <is>
-          <t>10th</t>
+          <t>13th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -6559,96 +6623,108 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>31.2</v>
+        <v>11.1</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>34.167</v>
+        <v>10.967</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>34.5</v>
+        <v>10.15</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>32.867</v>
+        <v>9.933</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>31.2</v>
+        <v>11.1</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="H90" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>11.4</v>
+      </c>
+      <c r="H90" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
-      <c r="J90" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K90" s="32" t="n">
-        <v>30</v>
-      </c>
-      <c r="L90" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="M90" s="32" t="n">
-        <v>33.615</v>
-      </c>
-      <c r="N90" s="32" t="n">
-        <v>33.444</v>
-      </c>
-      <c r="O90" s="32" t="n">
-        <v>32.893</v>
-      </c>
-      <c r="P90" s="32" t="n">
-        <v>32.75</v>
+      <c r="J90" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P90" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B91" s="32" t="n">
-        <v>17.7</v>
+        <v>12.6</v>
       </c>
       <c r="C91" s="32" t="n">
-        <v>19.933</v>
+        <v>12.267</v>
       </c>
       <c r="D91" s="32" t="n">
-        <v>18.9</v>
+        <v>12.5</v>
       </c>
       <c r="E91" s="32" t="n">
-        <v>17.867</v>
+        <v>12.733</v>
       </c>
       <c r="F91" s="32" t="n">
-        <v>17.7</v>
+        <v>12.6</v>
       </c>
       <c r="G91" s="32" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="H91" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>13.4</v>
+      </c>
+      <c r="H91" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I91" s="32" t="inlineStr"/>
@@ -6689,269 +6765,253 @@
       </c>
       <c r="Q91" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B92" s="32" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="C92" s="32" t="n">
-        <v>10.967</v>
-      </c>
-      <c r="D92" s="32" t="n">
-        <v>10.15</v>
-      </c>
-      <c r="E92" s="32" t="n">
-        <v>9.933</v>
-      </c>
-      <c r="F92" s="32" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="G92" s="32" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="H92" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="I92" s="32" t="inlineStr"/>
-      <c r="J92" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q92" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TOV</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="31" t="inlineStr">
-        <is>
-          <t>TOV</t>
-        </is>
-      </c>
-      <c r="B93" s="32" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="C93" s="32" t="n">
-        <v>12.267</v>
-      </c>
-      <c r="D93" s="32" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="E93" s="32" t="n">
-        <v>12.733</v>
-      </c>
-      <c r="F93" s="32" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="G93" s="32" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="H93" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I93" s="32" t="inlineStr"/>
-      <c r="J93" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q93" s="34" t="inlineStr">
-        <is>
-          <t>Opp TOV</t>
+      <c r="A93" s="29" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B94" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C94" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D94" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F94" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G94" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H94" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I94" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J94" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K94" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L94" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M94" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N94" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O94" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P94" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q94" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="29" t="inlineStr">
-        <is>
-          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
+      <c r="A95" s="31" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="C95" s="32" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="D95" s="32" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="E95" s="32" t="n">
+        <v>85.867</v>
+      </c>
+      <c r="F95" s="32" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="G95" s="32" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="H95" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J95" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K95" s="32" t="n">
+        <v>89.8</v>
+      </c>
+      <c r="L95" s="32" t="n">
+        <v>86.77800000000001</v>
+      </c>
+      <c r="M95" s="32" t="n">
+        <v>87.786</v>
+      </c>
+      <c r="N95" s="32" t="n">
+        <v>84.36799999999999</v>
+      </c>
+      <c r="O95" s="32" t="n">
+        <v>82.655</v>
+      </c>
+      <c r="P95" s="32" t="n">
+        <v>86.77800000000001</v>
+      </c>
+      <c r="Q95" s="34" t="inlineStr">
+        <is>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B96" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C96" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D96" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E96" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F96" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G96" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H96" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I96" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J96" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K96" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L96" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M96" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N96" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O96" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P96" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q96" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A96" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B96" s="32" t="n">
+        <v>109.659</v>
+      </c>
+      <c r="C96" s="32" t="n">
+        <v>107.942</v>
+      </c>
+      <c r="D96" s="32" t="n">
+        <v>105.587</v>
+      </c>
+      <c r="E96" s="32" t="n">
+        <v>105.509</v>
+      </c>
+      <c r="F96" s="32" t="n">
+        <v>109.659</v>
+      </c>
+      <c r="G96" s="32" t="n">
+        <v>115.565</v>
+      </c>
+      <c r="H96" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I96" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J96" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K96" s="32" t="n">
+        <v>113.552</v>
+      </c>
+      <c r="L96" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="M96" s="32" t="n">
+        <v>109.197</v>
+      </c>
+      <c r="N96" s="32" t="n">
+        <v>104.078</v>
+      </c>
+      <c r="O96" s="32" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="P96" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="Q96" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B97" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C97" s="32" t="n">
-        <v>85.2</v>
+        <v>0.544</v>
       </c>
       <c r="D97" s="32" t="n">
-        <v>84.90000000000001</v>
+        <v>0.533</v>
       </c>
       <c r="E97" s="32" t="n">
-        <v>85.867</v>
+        <v>0.535</v>
       </c>
       <c r="F97" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="G97" s="32" t="n">
-        <v>94.2</v>
+        <v>0.579</v>
       </c>
       <c r="H97" s="33" t="inlineStr">
         <is>
@@ -6969,52 +7029,52 @@
         </is>
       </c>
       <c r="K97" s="32" t="n">
-        <v>89.8</v>
+        <v>0.571</v>
       </c>
       <c r="L97" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>0.545</v>
       </c>
       <c r="M97" s="32" t="n">
-        <v>87.786</v>
+        <v>0.53</v>
       </c>
       <c r="N97" s="32" t="n">
-        <v>84.36799999999999</v>
+        <v>0.506</v>
       </c>
       <c r="O97" s="32" t="n">
-        <v>82.655</v>
+        <v>0.5</v>
       </c>
       <c r="P97" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>0.545</v>
       </c>
       <c r="Q97" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B98" s="32" t="n">
-        <v>109.659</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="C98" s="32" t="n">
-        <v>107.942</v>
+        <v>0.534</v>
       </c>
       <c r="D98" s="32" t="n">
-        <v>105.587</v>
+        <v>0.543</v>
       </c>
       <c r="E98" s="32" t="n">
-        <v>105.509</v>
+        <v>0.549</v>
       </c>
       <c r="F98" s="32" t="n">
-        <v>109.659</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="G98" s="32" t="n">
-        <v>115.565</v>
+        <v>0.582</v>
       </c>
       <c r="H98" s="33" t="inlineStr">
         <is>
@@ -7023,65 +7083,65 @@
       </c>
       <c r="I98" s="32" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="J98" s="36" t="inlineStr">
         <is>
-          <t>14th</t>
+          <t>10th</t>
         </is>
       </c>
       <c r="K98" s="32" t="n">
-        <v>113.552</v>
+        <v>0.5</v>
       </c>
       <c r="L98" s="32" t="n">
-        <v>108.265</v>
+        <v>0.514</v>
       </c>
       <c r="M98" s="32" t="n">
-        <v>109.197</v>
+        <v>0.5</v>
       </c>
       <c r="N98" s="32" t="n">
-        <v>104.078</v>
+        <v>0.494</v>
       </c>
       <c r="O98" s="32" t="n">
-        <v>102.45</v>
+        <v>0.497</v>
       </c>
       <c r="P98" s="32" t="n">
-        <v>108.265</v>
+        <v>0.514</v>
       </c>
       <c r="Q98" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.373</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>0.544</v>
+        <v>0.374</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>0.533</v>
+        <v>0.343</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>0.535</v>
+        <v>0.347</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.373</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>0.579</v>
+        <v>0.382</v>
       </c>
       <c r="H99" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I99" s="32" t="inlineStr">
@@ -7095,182 +7155,198 @@
         </is>
       </c>
       <c r="K99" s="32" t="n">
-        <v>0.571</v>
+        <v>0.453</v>
       </c>
       <c r="L99" s="32" t="n">
-        <v>0.545</v>
+        <v>0.39</v>
       </c>
       <c r="M99" s="32" t="n">
-        <v>0.53</v>
+        <v>0.381</v>
       </c>
       <c r="N99" s="32" t="n">
-        <v>0.506</v>
+        <v>0.347</v>
       </c>
       <c r="O99" s="32" t="n">
-        <v>0.5</v>
+        <v>0.337</v>
       </c>
       <c r="P99" s="32" t="n">
-        <v>0.545</v>
+        <v>0.39</v>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.767</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>0.534</v>
+        <v>0.744</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>0.543</v>
+        <v>0.749</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>0.549</v>
+        <v>0.779</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.767</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>0.582</v>
+        <v>0.842</v>
       </c>
       <c r="H100" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I100" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J100" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K100" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L100" s="32" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="M100" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N100" s="32" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="O100" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="P100" s="32" t="n">
-        <v>0.514</v>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I100" s="32" t="inlineStr"/>
+      <c r="J100" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>0.373</v>
+        <v>81.724</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>0.374</v>
+        <v>79.247</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>0.343</v>
+        <v>80.62</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>0.347</v>
+        <v>81.736</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>0.373</v>
+        <v>81.724</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>0.382</v>
-      </c>
-      <c r="H101" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I101" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J101" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K101" s="32" t="n">
-        <v>0.453</v>
-      </c>
-      <c r="L101" s="32" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="M101" s="32" t="n">
-        <v>0.381</v>
-      </c>
-      <c r="N101" s="32" t="n">
-        <v>0.347</v>
-      </c>
-      <c r="O101" s="32" t="n">
-        <v>0.337</v>
-      </c>
-      <c r="P101" s="32" t="n">
-        <v>0.39</v>
+        <v>82.304</v>
+      </c>
+      <c r="H101" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I101" s="32" t="inlineStr"/>
+      <c r="J101" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
-        <v>0.767</v>
+        <v>0.591</v>
       </c>
       <c r="C102" s="32" t="n">
-        <v>0.744</v>
+        <v>0.57</v>
       </c>
       <c r="D102" s="32" t="n">
-        <v>0.749</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="E102" s="32" t="n">
-        <v>0.779</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F102" s="32" t="n">
-        <v>0.767</v>
+        <v>0.591</v>
       </c>
       <c r="G102" s="32" t="n">
-        <v>0.842</v>
+        <v>0.613</v>
       </c>
       <c r="H102" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I102" s="32" t="inlineStr"/>
@@ -7311,37 +7387,37 @@
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>81.724</v>
+        <v>0.265</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>79.247</v>
+        <v>0.255</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>80.62</v>
+        <v>0.253</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>81.736</v>
+        <v>0.245</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>81.724</v>
+        <v>0.265</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>82.304</v>
-      </c>
-      <c r="H103" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
+        <v>0.287</v>
+      </c>
+      <c r="H103" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I103" s="32" t="inlineStr"/>
@@ -7382,108 +7458,100 @@
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>0.591</v>
+        <v>37.6</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>0.57</v>
+        <v>34.9</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>0.5610000000000001</v>
+        <v>36.05</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>0.5649999999999999</v>
+        <v>36.467</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>0.591</v>
+        <v>37.6</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>0.613</v>
+        <v>40.4</v>
       </c>
       <c r="H104" s="33" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I104" s="32" t="inlineStr"/>
-      <c r="J104" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P104" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I104" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J104" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K104" s="32" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="L104" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="M104" s="32" t="n">
+        <v>34.929</v>
+      </c>
+      <c r="N104" s="32" t="n">
+        <v>35.053</v>
+      </c>
+      <c r="O104" s="32" t="n">
+        <v>35.69</v>
+      </c>
+      <c r="P104" s="32" t="n">
+        <v>34.556</v>
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>0.265</v>
+        <v>21.1</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>0.255</v>
+        <v>21.533</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>0.253</v>
+        <v>21.1</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>0.245</v>
+        <v>20.867</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>0.265</v>
+        <v>21.1</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>0.287</v>
+        <v>23.2</v>
       </c>
       <c r="H105" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -7524,100 +7592,108 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>37.6</v>
+        <v>13</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>34.9</v>
+        <v>12.567</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>36.05</v>
+        <v>13.05</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>36.467</v>
+        <v>12.867</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>37.6</v>
+        <v>13</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>40.4</v>
+        <v>14.2</v>
       </c>
       <c r="H106" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I106" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J106" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K106" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="L106" s="32" t="n">
-        <v>34.556</v>
-      </c>
-      <c r="M106" s="32" t="n">
-        <v>34.929</v>
-      </c>
-      <c r="N106" s="32" t="n">
-        <v>35.053</v>
-      </c>
-      <c r="O106" s="32" t="n">
-        <v>35.69</v>
-      </c>
-      <c r="P106" s="32" t="n">
-        <v>34.556</v>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I106" s="32" t="inlineStr"/>
+      <c r="J106" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P106" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q106" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B107" s="32" t="n">
-        <v>21.1</v>
+        <v>14.8</v>
       </c>
       <c r="C107" s="32" t="n">
-        <v>21.533</v>
+        <v>12.733</v>
       </c>
       <c r="D107" s="32" t="n">
-        <v>21.1</v>
+        <v>13.35</v>
       </c>
       <c r="E107" s="32" t="n">
-        <v>20.867</v>
+        <v>13.733</v>
       </c>
       <c r="F107" s="32" t="n">
-        <v>21.1</v>
+        <v>14.8</v>
       </c>
       <c r="G107" s="32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="H107" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
+        <v>14.4</v>
+      </c>
+      <c r="H107" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
         </is>
       </c>
       <c r="I107" s="32" t="inlineStr"/>
@@ -7657,148 +7733,6 @@
         </is>
       </c>
       <c r="Q107" s="34" t="inlineStr">
-        <is>
-          <t>Opp AST</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B108" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="C108" s="32" t="n">
-        <v>12.567</v>
-      </c>
-      <c r="D108" s="32" t="n">
-        <v>13.05</v>
-      </c>
-      <c r="E108" s="32" t="n">
-        <v>12.867</v>
-      </c>
-      <c r="F108" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="G108" s="32" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="H108" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I108" s="32" t="inlineStr"/>
-      <c r="J108" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q108" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="31" t="inlineStr">
-        <is>
-          <t>TOV</t>
-        </is>
-      </c>
-      <c r="B109" s="32" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="C109" s="32" t="n">
-        <v>12.733</v>
-      </c>
-      <c r="D109" s="32" t="n">
-        <v>13.35</v>
-      </c>
-      <c r="E109" s="32" t="n">
-        <v>13.733</v>
-      </c>
-      <c r="F109" s="32" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="G109" s="32" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H109" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
-        </is>
-      </c>
-      <c r="I109" s="32" t="inlineStr"/>
-      <c r="J109" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q109" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>

</xml_diff>

<commit_message>
data: hourly update 2026-07-14 00:02Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-13.xlsx
+++ b/data/output/workbook/2026-07-13.xlsx
@@ -363,7 +363,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12306300"/>
+    <ext cx="10125075" cy="12877800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13 19:02</t>
+          <t>2026-07-13 20:02</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1123,22 +1123,22 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5632</v>
+        <v>0.5389</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-129</v>
+        <v>-117</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1189,22 +1189,22 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Over 171.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5389</v>
+        <v>0.5495</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-117</v>
+        <v>-122</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1306,37 +1306,37 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Minnesota Lynx</t>
+          <t>Washington Mystics @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 169.5</t>
+          <t>Toronto Tempo +0.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5162</v>
+        <v>0.54</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-107</v>
+        <v>-117</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>-106</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1369,9 +1369,75 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Over 169.5</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>0.5247000000000001</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>-104</v>
+      </c>
+      <c r="I9" s="13">
+        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
+        <v/>
+      </c>
+      <c r="K9" s="17">
+        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L9" s="18">
+        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M9" s="12">
+        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Model 52.5% (fair -110). Your call.</t>
+        </is>
+      </c>
+      <c r="O9" s="15" t="n"/>
+      <c r="P9" s="16">
+        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J8">
+  <conditionalFormatting sqref="J5:J9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1944,7 +2010,7 @@
         <v>106</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -2010,7 +2076,7 @@
         <v>-106</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2066,17 +2132,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream -9.5</t>
+          <t>Atlanta Dream -10.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3905243127429648</v>
+        <v>0.3606608556669979</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>104</v>
+        <v>-102</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2100,7 +2166,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +156). Your call.</t>
+          <t>Model 36.1% (fair +177). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -2132,17 +2198,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks +9.5</t>
+          <t>Los Angeles Sparks +10.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6094756872570352</v>
+        <v>0.6393391443330021</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-156</v>
+        <v>-177</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2166,7 +2232,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 63.9% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -2334,13 +2400,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5162</v>
+        <v>0.5247000000000001</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-107</v>
+        <v>-110</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2364,7 +2430,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 52.5% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2400,13 +2466,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4838</v>
+        <v>0.4752999999999999</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -2430,7 +2496,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 47.5% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2472,7 +2538,7 @@
         <v>102</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -2538,7 +2604,7 @@
         <v>-102</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>100</v>
+        <v>-105</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -2726,17 +2792,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.7045896324040164</v>
+        <v>0.7245695517138792</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-239</v>
+        <v>-263</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -2760,7 +2826,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 70.5% (fair -239). Your call.</t>
+          <t>Model 72.5% (fair -263). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -2792,17 +2858,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 168.5</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.2954103675959836</v>
+        <v>0.2754304482861208</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>239</v>
+        <v>263</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -2826,7 +2892,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 29.5% (fair +239). Your call.</t>
+          <t>Model 27.5% (fair +263). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -2868,7 +2934,7 @@
         <v>103</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -3122,17 +3188,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 170.5</t>
+          <t>Over 171.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5632</v>
+        <v>0.5495</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-129</v>
+        <v>-122</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -3156,7 +3222,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -3188,14 +3254,14 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 170.5</t>
+          <t>Under 171.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4368</v>
+        <v>0.4505</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>108</v>
@@ -3222,7 +3288,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -3254,17 +3320,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo -1.5</t>
+          <t>Toronto Tempo +0.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5051</v>
+        <v>0.54</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-102</v>
+        <v>-117</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>100</v>
+        <v>-106</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -3288,7 +3354,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -3320,14 +3386,14 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics +1.5</t>
+          <t>Washington Mystics -0.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4949</v>
+        <v>0.46</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>104</v>
@@ -3354,7 +3420,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -5807,7 +5873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q107"/>
+  <dimension ref="A1:Q111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5824,765 +5890,493 @@
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="29" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
         <is>
           <t>Phoenix Mercury offense vs Minnesota Lynx defense</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="30" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B78" s="30" t="inlineStr">
+      <c r="B82" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C78" s="30" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D78" s="30" t="inlineStr">
+      <c r="D82" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E78" s="30" t="inlineStr">
+      <c r="E82" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F78" s="30" t="inlineStr">
+      <c r="F82" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G78" s="30" t="inlineStr">
+      <c r="G82" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H78" s="30" t="inlineStr">
+      <c r="H82" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I78" s="30" t="inlineStr">
+      <c r="I82" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J78" s="30" t="inlineStr">
+      <c r="J82" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K78" s="30" t="inlineStr">
+      <c r="K82" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L78" s="30" t="inlineStr">
+      <c r="L82" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M78" s="30" t="inlineStr">
+      <c r="M82" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N78" s="30" t="inlineStr">
+      <c r="N82" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O78" s="30" t="inlineStr">
+      <c r="O82" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P78" s="30" t="inlineStr">
+      <c r="P82" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q78" s="30" t="inlineStr">
+      <c r="Q82" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="31" t="inlineStr">
-        <is>
-          <t>PPG</t>
-        </is>
-      </c>
-      <c r="B79" s="32" t="n">
-        <v>83</v>
-      </c>
-      <c r="C79" s="32" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="D79" s="32" t="n">
-        <v>83.05</v>
-      </c>
-      <c r="E79" s="32" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="F79" s="32" t="n">
-        <v>83</v>
-      </c>
-      <c r="G79" s="32" t="n">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="H79" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="n">
-        <v>72.75</v>
-      </c>
-      <c r="L79" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="M79" s="32" t="n">
-        <v>80</v>
-      </c>
-      <c r="N79" s="32" t="n">
-        <v>78.72199999999999</v>
-      </c>
-      <c r="O79" s="32" t="n">
-        <v>79</v>
-      </c>
-      <c r="P79" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="Q79" s="34" t="inlineStr">
-        <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B80" s="32" t="n">
-        <v>101.929</v>
-      </c>
-      <c r="C80" s="32" t="n">
-        <v>102.13</v>
-      </c>
-      <c r="D80" s="32" t="n">
-        <v>101.973</v>
-      </c>
-      <c r="E80" s="32" t="n">
-        <v>102.639</v>
-      </c>
-      <c r="F80" s="32" t="n">
-        <v>101.929</v>
-      </c>
-      <c r="G80" s="32" t="n">
-        <v>97.006</v>
-      </c>
-      <c r="H80" s="36" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I80" s="32" t="inlineStr"/>
-      <c r="J80" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K80" s="32" t="n">
-        <v>88.01600000000001</v>
-      </c>
-      <c r="L80" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="M80" s="32" t="n">
-        <v>97.129</v>
-      </c>
-      <c r="N80" s="32" t="n">
-        <v>96.706</v>
-      </c>
-      <c r="O80" s="32" t="n">
-        <v>98.628</v>
-      </c>
-      <c r="P80" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="Q80" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B81" s="32" t="n">
-        <v>0.476</v>
-      </c>
-      <c r="C81" s="32" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="D81" s="32" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="E81" s="32" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="F81" s="32" t="n">
-        <v>0.476</v>
-      </c>
-      <c r="G81" s="32" t="n">
-        <v>0.453</v>
-      </c>
-      <c r="H81" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K81" s="32" t="n">
-        <v>0.408</v>
-      </c>
-      <c r="L81" s="32" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="M81" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="N81" s="32" t="n">
-        <v>0.464</v>
-      </c>
-      <c r="O81" s="32" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="P81" s="32" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="Q81" s="34" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="31" t="inlineStr">
-        <is>
-          <t>2PT%</t>
-        </is>
-      </c>
-      <c r="B82" s="32" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="C82" s="32" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="D82" s="32" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="E82" s="32" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="F82" s="32" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="G82" s="32" t="n">
-        <v>0.454</v>
-      </c>
-      <c r="H82" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="L82" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="M82" s="32" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="N82" s="32" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="O82" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="P82" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="Q82" s="34" t="inlineStr">
-        <is>
-          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>0.32</v>
+        <v>83</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>0.33</v>
+        <v>82.3</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>0.315</v>
+        <v>83.05</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>0.318</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>0.32</v>
+        <v>83</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>0.293</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="H83" s="36" t="inlineStr">
         <is>
-          <t>12th</t>
+          <t>11th</t>
         </is>
       </c>
       <c r="I83" s="32" t="inlineStr"/>
       <c r="J83" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="K83" s="32" t="n">
-        <v>0.275</v>
+        <v>72.75</v>
       </c>
       <c r="L83" s="32" t="n">
-        <v>0.281</v>
+        <v>79.75</v>
       </c>
       <c r="M83" s="32" t="n">
-        <v>0.308</v>
+        <v>80</v>
       </c>
       <c r="N83" s="32" t="n">
-        <v>0.311</v>
+        <v>78.72199999999999</v>
       </c>
       <c r="O83" s="32" t="n">
-        <v>0.342</v>
+        <v>79</v>
       </c>
       <c r="P83" s="32" t="n">
-        <v>0.281</v>
+        <v>79.75</v>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>101.929</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>0.797</v>
+        <v>102.13</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>0.822</v>
+        <v>101.973</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>0.8070000000000001</v>
+        <v>102.639</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>0.8129999999999999</v>
+        <v>101.929</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="H84" s="33" t="inlineStr">
-        <is>
-          <t>4th</t>
+        <v>97.006</v>
+      </c>
+      <c r="H84" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
-      <c r="J84" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J84" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K84" s="32" t="n">
+        <v>88.01600000000001</v>
+      </c>
+      <c r="L84" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="M84" s="32" t="n">
+        <v>97.129</v>
+      </c>
+      <c r="N84" s="32" t="n">
+        <v>96.706</v>
+      </c>
+      <c r="O84" s="32" t="n">
+        <v>98.628</v>
+      </c>
+      <c r="P84" s="32" t="n">
+        <v>95.66500000000001</v>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.476</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>80.69199999999999</v>
+        <v>0.491</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>81.45399999999999</v>
+        <v>0.486</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>81.39700000000001</v>
+        <v>0.488</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>81.31999999999999</v>
+        <v>0.476</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>79.672</v>
-      </c>
-      <c r="H85" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
+        <v>0.453</v>
+      </c>
+      <c r="H85" s="36" t="inlineStr">
+        <is>
+          <t>12th</t>
         </is>
       </c>
       <c r="I85" s="32" t="inlineStr"/>
-      <c r="J85" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J85" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K85" s="32" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="L85" s="32" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="M85" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="N85" s="32" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="O85" s="32" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="P85" s="32" t="n">
+        <v>0.441</v>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.543</v>
+        <v>0.467</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.54</v>
+        <v>0.48</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.54</v>
+        <v>0.486</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.547</v>
+        <v>0.488</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.543</v>
+        <v>0.467</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.519</v>
+        <v>0.454</v>
       </c>
       <c r="H86" s="36" t="inlineStr">
         <is>
-          <t>11th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
-      <c r="J86" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J86" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K86" s="32" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="L86" s="32" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="M86" s="32" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="N86" s="32" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="O86" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="P86" s="32" t="n">
+        <v>0.449</v>
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>0.225</v>
+        <v>0.32</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>0.228</v>
+        <v>0.33</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>0.231</v>
+        <v>0.315</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>0.226</v>
+        <v>0.318</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>0.225</v>
+        <v>0.32</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>0.231</v>
+        <v>0.293</v>
       </c>
       <c r="H87" s="36" t="inlineStr">
         <is>
-          <t>10th</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
-      <c r="J87" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J87" s="33" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K87" s="32" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="L87" s="32" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="M87" s="32" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="N87" s="32" t="n">
+        <v>0.311</v>
+      </c>
+      <c r="O87" s="32" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="P87" s="32" t="n">
+        <v>0.281</v>
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>31.2</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>34.167</v>
+        <v>0.797</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>34.5</v>
+        <v>0.822</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>32.867</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>31.2</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="H88" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>0.821</v>
+      </c>
+      <c r="H88" s="33" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
-      <c r="J88" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K88" s="32" t="n">
-        <v>30</v>
-      </c>
-      <c r="L88" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="M88" s="32" t="n">
-        <v>33.615</v>
-      </c>
-      <c r="N88" s="32" t="n">
-        <v>33.444</v>
-      </c>
-      <c r="O88" s="32" t="n">
-        <v>32.893</v>
-      </c>
-      <c r="P88" s="32" t="n">
-        <v>32.75</v>
+      <c r="J88" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>17.7</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>19.933</v>
+        <v>80.69199999999999</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>18.9</v>
+        <v>81.45399999999999</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>17.867</v>
+        <v>81.39700000000001</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>17.7</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="H89" s="36" t="inlineStr">
-        <is>
-          <t>13th</t>
+        <v>79.672</v>
+      </c>
+      <c r="H89" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -6623,37 +6417,37 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>11.1</v>
+        <v>0.543</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>10.967</v>
+        <v>0.54</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>10.15</v>
+        <v>0.54</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>9.933</v>
+        <v>0.547</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>11.1</v>
+        <v>0.543</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="H90" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
+        <v>0.519</v>
+      </c>
+      <c r="H90" s="36" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
@@ -6694,37 +6488,37 @@
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B91" s="32" t="n">
-        <v>12.6</v>
+        <v>0.225</v>
       </c>
       <c r="C91" s="32" t="n">
-        <v>12.267</v>
+        <v>0.228</v>
       </c>
       <c r="D91" s="32" t="n">
-        <v>12.5</v>
+        <v>0.231</v>
       </c>
       <c r="E91" s="32" t="n">
-        <v>12.733</v>
+        <v>0.226</v>
       </c>
       <c r="F91" s="32" t="n">
-        <v>12.6</v>
+        <v>0.225</v>
       </c>
       <c r="G91" s="32" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="H91" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
+        <v>0.231</v>
+      </c>
+      <c r="H91" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
         </is>
       </c>
       <c r="I91" s="32" t="inlineStr"/>
@@ -6765,383 +6559,403 @@
       </c>
       <c r="Q91" s="34" t="inlineStr">
         <is>
-          <t>Opp TOV</t>
+          <t>Opp OREB%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="B92" s="32" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="C92" s="32" t="n">
+        <v>34.167</v>
+      </c>
+      <c r="D92" s="32" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="E92" s="32" t="n">
+        <v>32.867</v>
+      </c>
+      <c r="F92" s="32" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="G92" s="32" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="H92" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
+        </is>
+      </c>
+      <c r="I92" s="32" t="inlineStr"/>
+      <c r="J92" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K92" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="L92" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="M92" s="32" t="n">
+        <v>33.615</v>
+      </c>
+      <c r="N92" s="32" t="n">
+        <v>33.444</v>
+      </c>
+      <c r="O92" s="32" t="n">
+        <v>32.893</v>
+      </c>
+      <c r="P92" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="Q92" s="34" t="inlineStr">
+        <is>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="29" t="inlineStr">
-        <is>
-          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
+      <c r="A93" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="C93" s="32" t="n">
+        <v>19.933</v>
+      </c>
+      <c r="D93" s="32" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="E93" s="32" t="n">
+        <v>17.867</v>
+      </c>
+      <c r="F93" s="32" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G93" s="32" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="H93" s="36" t="inlineStr">
+        <is>
+          <t>13th</t>
+        </is>
+      </c>
+      <c r="I93" s="32" t="inlineStr"/>
+      <c r="J93" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q93" s="34" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B94" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C94" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D94" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E94" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F94" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G94" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H94" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I94" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J94" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K94" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L94" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M94" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N94" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O94" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P94" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q94" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A94" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B94" s="32" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C94" s="32" t="n">
+        <v>10.967</v>
+      </c>
+      <c r="D94" s="32" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="E94" s="32" t="n">
+        <v>9.933</v>
+      </c>
+      <c r="F94" s="32" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="G94" s="32" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H94" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="I94" s="32" t="inlineStr"/>
+      <c r="J94" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q94" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B95" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="C95" s="32" t="n">
-        <v>85.2</v>
+        <v>12.267</v>
       </c>
       <c r="D95" s="32" t="n">
-        <v>84.90000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="E95" s="32" t="n">
-        <v>85.867</v>
+        <v>12.733</v>
       </c>
       <c r="F95" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="G95" s="32" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="H95" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I95" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J95" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K95" s="32" t="n">
-        <v>89.8</v>
-      </c>
-      <c r="L95" s="32" t="n">
-        <v>86.77800000000001</v>
-      </c>
-      <c r="M95" s="32" t="n">
-        <v>87.786</v>
-      </c>
-      <c r="N95" s="32" t="n">
-        <v>84.36799999999999</v>
-      </c>
-      <c r="O95" s="32" t="n">
-        <v>82.655</v>
-      </c>
-      <c r="P95" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>13.4</v>
+      </c>
+      <c r="H95" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="inlineStr"/>
+      <c r="J95" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q95" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B96" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="C96" s="32" t="n">
-        <v>107.942</v>
-      </c>
-      <c r="D96" s="32" t="n">
-        <v>105.587</v>
-      </c>
-      <c r="E96" s="32" t="n">
-        <v>105.509</v>
-      </c>
-      <c r="F96" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="G96" s="32" t="n">
-        <v>115.565</v>
-      </c>
-      <c r="H96" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I96" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J96" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K96" s="32" t="n">
-        <v>113.552</v>
-      </c>
-      <c r="L96" s="32" t="n">
-        <v>108.265</v>
-      </c>
-      <c r="M96" s="32" t="n">
-        <v>109.197</v>
-      </c>
-      <c r="N96" s="32" t="n">
-        <v>104.078</v>
-      </c>
-      <c r="O96" s="32" t="n">
-        <v>102.45</v>
-      </c>
-      <c r="P96" s="32" t="n">
-        <v>108.265</v>
-      </c>
-      <c r="Q96" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp TOV</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B97" s="32" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="C97" s="32" t="n">
-        <v>0.544</v>
-      </c>
-      <c r="D97" s="32" t="n">
-        <v>0.533</v>
-      </c>
-      <c r="E97" s="32" t="n">
-        <v>0.535</v>
-      </c>
-      <c r="F97" s="32" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="G97" s="32" t="n">
-        <v>0.579</v>
-      </c>
-      <c r="H97" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I97" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J97" s="36" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K97" s="32" t="n">
-        <v>0.571</v>
-      </c>
-      <c r="L97" s="32" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="M97" s="32" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N97" s="32" t="n">
-        <v>0.506</v>
-      </c>
-      <c r="O97" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P97" s="32" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="Q97" s="34" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx offense vs Phoenix Mercury defense</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="31" t="inlineStr">
-        <is>
-          <t>2PT%</t>
-        </is>
-      </c>
-      <c r="B98" s="32" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="C98" s="32" t="n">
-        <v>0.534</v>
-      </c>
-      <c r="D98" s="32" t="n">
-        <v>0.543</v>
-      </c>
-      <c r="E98" s="32" t="n">
-        <v>0.549</v>
-      </c>
-      <c r="F98" s="32" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="G98" s="32" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="H98" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I98" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J98" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K98" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L98" s="32" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="M98" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N98" s="32" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="O98" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="P98" s="32" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="Q98" s="34" t="inlineStr">
-        <is>
-          <t>Opp 2PT%</t>
+      <c r="A98" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B98" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C98" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D98" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E98" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F98" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G98" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H98" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I98" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J98" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K98" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L98" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M98" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N98" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O98" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P98" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q98" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>0.373</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>0.374</v>
+        <v>85.2</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>0.343</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>0.347</v>
+        <v>85.867</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>0.373</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>0.382</v>
+        <v>94.2</v>
       </c>
       <c r="H99" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I99" s="32" t="inlineStr">
@@ -7155,403 +6969,379 @@
         </is>
       </c>
       <c r="K99" s="32" t="n">
-        <v>0.453</v>
+        <v>89.8</v>
       </c>
       <c r="L99" s="32" t="n">
-        <v>0.39</v>
+        <v>86.77800000000001</v>
       </c>
       <c r="M99" s="32" t="n">
-        <v>0.381</v>
+        <v>87.786</v>
       </c>
       <c r="N99" s="32" t="n">
-        <v>0.347</v>
+        <v>84.36799999999999</v>
       </c>
       <c r="O99" s="32" t="n">
-        <v>0.337</v>
+        <v>82.655</v>
       </c>
       <c r="P99" s="32" t="n">
-        <v>0.39</v>
+        <v>86.77800000000001</v>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>0.767</v>
+        <v>109.659</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>0.744</v>
+        <v>107.942</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>0.749</v>
+        <v>105.587</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>0.779</v>
+        <v>105.509</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>0.767</v>
+        <v>109.659</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>0.842</v>
+        <v>115.565</v>
       </c>
       <c r="H100" s="33" t="inlineStr">
         <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="I100" s="32" t="inlineStr"/>
-      <c r="J100" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I100" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J100" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K100" s="32" t="n">
+        <v>113.552</v>
+      </c>
+      <c r="L100" s="32" t="n">
+        <v>108.265</v>
+      </c>
+      <c r="M100" s="32" t="n">
+        <v>109.197</v>
+      </c>
+      <c r="N100" s="32" t="n">
+        <v>104.078</v>
+      </c>
+      <c r="O100" s="32" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="P100" s="32" t="n">
+        <v>108.265</v>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>81.724</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>79.247</v>
+        <v>0.544</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>80.62</v>
+        <v>0.533</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>81.736</v>
+        <v>0.535</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>81.724</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>82.304</v>
-      </c>
-      <c r="H101" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I101" s="32" t="inlineStr"/>
-      <c r="J101" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.579</v>
+      </c>
+      <c r="H101" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I101" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J101" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K101" s="32" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="L101" s="32" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="M101" s="32" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N101" s="32" t="n">
+        <v>0.506</v>
+      </c>
+      <c r="O101" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P101" s="32" t="n">
+        <v>0.545</v>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
-        <v>0.591</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="C102" s="32" t="n">
-        <v>0.57</v>
+        <v>0.534</v>
       </c>
       <c r="D102" s="32" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E102" s="32" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="F102" s="32" t="n">
         <v>0.5610000000000001</v>
       </c>
-      <c r="E102" s="32" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="F102" s="32" t="n">
-        <v>0.591</v>
-      </c>
       <c r="G102" s="32" t="n">
-        <v>0.613</v>
+        <v>0.582</v>
       </c>
       <c r="H102" s="33" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I102" s="32" t="inlineStr"/>
-      <c r="J102" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I102" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J102" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K102" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L102" s="32" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="M102" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N102" s="32" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="O102" s="32" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="P102" s="32" t="n">
+        <v>0.514</v>
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>0.265</v>
+        <v>0.373</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>0.255</v>
+        <v>0.374</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>0.253</v>
+        <v>0.343</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>0.245</v>
+        <v>0.347</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>0.265</v>
+        <v>0.373</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>0.287</v>
+        <v>0.382</v>
       </c>
       <c r="H103" s="33" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="I103" s="32" t="inlineStr"/>
-      <c r="J103" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I103" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J103" s="36" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K103" s="32" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="L103" s="32" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="M103" s="32" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="N103" s="32" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="O103" s="32" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="P103" s="32" t="n">
+        <v>0.39</v>
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>37.6</v>
+        <v>0.767</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>34.9</v>
+        <v>0.744</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>36.05</v>
+        <v>0.749</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>36.467</v>
+        <v>0.779</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>37.6</v>
+        <v>0.767</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>40.4</v>
+        <v>0.842</v>
       </c>
       <c r="H104" s="33" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I104" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J104" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K104" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="L104" s="32" t="n">
-        <v>34.556</v>
-      </c>
-      <c r="M104" s="32" t="n">
-        <v>34.929</v>
-      </c>
-      <c r="N104" s="32" t="n">
-        <v>35.053</v>
-      </c>
-      <c r="O104" s="32" t="n">
-        <v>35.69</v>
-      </c>
-      <c r="P104" s="32" t="n">
-        <v>34.556</v>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I104" s="32" t="inlineStr"/>
+      <c r="J104" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>21.1</v>
+        <v>81.724</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>21.533</v>
+        <v>79.247</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>21.1</v>
+        <v>80.62</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>20.867</v>
+        <v>81.736</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>21.1</v>
+        <v>81.724</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="H105" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
+        <v>82.304</v>
+      </c>
+      <c r="H105" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -7592,37 +7382,37 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>13</v>
+        <v>0.591</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>12.567</v>
+        <v>0.57</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>13.05</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>12.867</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>13</v>
+        <v>0.591</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>14.2</v>
+        <v>0.613</v>
       </c>
       <c r="H106" s="33" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I106" s="32" t="inlineStr"/>
@@ -7663,37 +7453,37 @@
       </c>
       <c r="Q106" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B107" s="32" t="n">
-        <v>14.8</v>
+        <v>0.265</v>
       </c>
       <c r="C107" s="32" t="n">
-        <v>12.733</v>
+        <v>0.255</v>
       </c>
       <c r="D107" s="32" t="n">
-        <v>13.35</v>
+        <v>0.253</v>
       </c>
       <c r="E107" s="32" t="n">
-        <v>13.733</v>
+        <v>0.245</v>
       </c>
       <c r="F107" s="32" t="n">
-        <v>14.8</v>
+        <v>0.265</v>
       </c>
       <c r="G107" s="32" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H107" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>0.287</v>
+      </c>
+      <c r="H107" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I107" s="32" t="inlineStr"/>
@@ -7733,6 +7523,282 @@
         </is>
       </c>
       <c r="Q107" s="34" t="inlineStr">
+        <is>
+          <t>Opp OREB%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="31" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="B108" s="32" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="C108" s="32" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="D108" s="32" t="n">
+        <v>36.05</v>
+      </c>
+      <c r="E108" s="32" t="n">
+        <v>36.467</v>
+      </c>
+      <c r="F108" s="32" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G108" s="32" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="H108" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I108" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J108" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K108" s="32" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="L108" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="M108" s="32" t="n">
+        <v>34.929</v>
+      </c>
+      <c r="N108" s="32" t="n">
+        <v>35.053</v>
+      </c>
+      <c r="O108" s="32" t="n">
+        <v>35.69</v>
+      </c>
+      <c r="P108" s="32" t="n">
+        <v>34.556</v>
+      </c>
+      <c r="Q108" s="34" t="inlineStr">
+        <is>
+          <t>Opp REB</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="C109" s="32" t="n">
+        <v>21.533</v>
+      </c>
+      <c r="D109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="E109" s="32" t="n">
+        <v>20.867</v>
+      </c>
+      <c r="F109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="G109" s="32" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="H109" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I109" s="32" t="inlineStr"/>
+      <c r="J109" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q109" s="34" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C110" s="32" t="n">
+        <v>12.567</v>
+      </c>
+      <c r="D110" s="32" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="E110" s="32" t="n">
+        <v>12.867</v>
+      </c>
+      <c r="F110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="G110" s="32" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H110" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I110" s="32" t="inlineStr"/>
+      <c r="J110" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q110" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="31" t="inlineStr">
+        <is>
+          <t>TOV</t>
+        </is>
+      </c>
+      <c r="B111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C111" s="32" t="n">
+        <v>12.733</v>
+      </c>
+      <c r="D111" s="32" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="E111" s="32" t="n">
+        <v>13.733</v>
+      </c>
+      <c r="F111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="G111" s="32" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H111" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I111" s="32" t="inlineStr"/>
+      <c r="J111" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q111" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>

</xml_diff>